<commit_message>
docs: update two business template Excel files
add new 交付工具模板表格 and update 行业案例模板表格
</commit_message>
<xml_diff>
--- a/template/业主考勤表模版.xlsx
+++ b/template/业主考勤表模版.xlsx
@@ -4,14 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="9060"/>
+    <workbookView windowWidth="22188" windowHeight="9060" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="考勤表" sheetId="3" r:id="rId1"/>
     <sheet name="工资表" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">工资表!$A$3:$Z$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">工资表!$A$3:$Z$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">考勤表!$A$1:$AL$38</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">工资表!$1:$3</definedName>
   </definedNames>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="70">
   <si>
     <t>中石化第四建设有限公司-中煤榆林煤炭深加工基地工程项目部-2026年5月打卡考勤表</t>
   </si>
@@ -234,12 +234,6 @@
   </si>
   <si>
     <t>102100000</t>
-  </si>
-  <si>
-    <t>小计</t>
-  </si>
-  <si>
-    <t>合计</t>
   </si>
   <si>
     <t>项目综合管理办公室：</t>
@@ -1225,7 +1219,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1279,12 +1273,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1773,1782 +1761,1782 @@
   <dimension ref="A1:AL38"/>
   <sheetFormatPr defaultColWidth="14.4833333333333" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="4.05833333333333" style="26" customWidth="1"/>
-    <col min="2" max="2" width="13.6" style="25" customWidth="1"/>
-    <col min="3" max="3" width="5.88333333333333" style="25" customWidth="1"/>
-    <col min="4" max="4" width="4.75" style="25" customWidth="1"/>
-    <col min="5" max="5" width="2.60833333333333" style="26" customWidth="1"/>
-    <col min="6" max="14" width="2.48333333333333" style="26" customWidth="1"/>
-    <col min="15" max="15" width="3.95833333333333" style="27" customWidth="1"/>
-    <col min="16" max="28" width="2.48333333333333" style="26" customWidth="1"/>
-    <col min="29" max="30" width="3.39166666666667" style="27" customWidth="1"/>
-    <col min="31" max="35" width="2.48333333333333" style="26" customWidth="1"/>
-    <col min="36" max="36" width="4.98333333333333" style="27" customWidth="1"/>
-    <col min="37" max="37" width="4.625" style="25" customWidth="1"/>
-    <col min="38" max="38" width="7.425" style="25" customWidth="1"/>
-    <col min="39" max="16384" width="14.4833333333333" style="25"/>
+    <col min="1" max="1" width="4.05833333333333" style="24" customWidth="1"/>
+    <col min="2" max="2" width="13.6" style="23" customWidth="1"/>
+    <col min="3" max="3" width="5.88333333333333" style="23" customWidth="1"/>
+    <col min="4" max="4" width="4.75" style="23" customWidth="1"/>
+    <col min="5" max="5" width="2.60833333333333" style="24" customWidth="1"/>
+    <col min="6" max="14" width="2.48333333333333" style="24" customWidth="1"/>
+    <col min="15" max="15" width="3.95833333333333" style="25" customWidth="1"/>
+    <col min="16" max="28" width="2.48333333333333" style="24" customWidth="1"/>
+    <col min="29" max="30" width="3.39166666666667" style="25" customWidth="1"/>
+    <col min="31" max="35" width="2.48333333333333" style="24" customWidth="1"/>
+    <col min="36" max="36" width="4.98333333333333" style="25" customWidth="1"/>
+    <col min="37" max="37" width="4.625" style="23" customWidth="1"/>
+    <col min="38" max="38" width="7.425" style="23" customWidth="1"/>
+    <col min="39" max="16384" width="14.4833333333333" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" s="25" customFormat="1" spans="1:38">
-      <c r="A1" s="28" t="s">
+    <row r="1" s="23" customFormat="1" spans="1:38">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="31"/>
-      <c r="P1" s="30"/>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="30"/>
-      <c r="V1" s="30"/>
-      <c r="W1" s="30"/>
-      <c r="X1" s="30"/>
-      <c r="Y1" s="30"/>
-      <c r="Z1" s="30"/>
-      <c r="AA1" s="30"/>
-      <c r="AB1" s="30"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="31"/>
-      <c r="AE1" s="30"/>
-      <c r="AF1" s="30"/>
-      <c r="AG1" s="30"/>
-      <c r="AH1" s="30"/>
-      <c r="AI1" s="30"/>
-      <c r="AJ1" s="31"/>
-      <c r="AK1" s="29"/>
-      <c r="AL1" s="32"/>
-    </row>
-    <row r="2" s="25" customFormat="1" spans="1:38">
-      <c r="A2" s="28" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
+      <c r="T1" s="28"/>
+      <c r="U1" s="28"/>
+      <c r="V1" s="28"/>
+      <c r="W1" s="28"/>
+      <c r="X1" s="28"/>
+      <c r="Y1" s="28"/>
+      <c r="Z1" s="28"/>
+      <c r="AA1" s="28"/>
+      <c r="AB1" s="28"/>
+      <c r="AC1" s="29"/>
+      <c r="AD1" s="29"/>
+      <c r="AE1" s="28"/>
+      <c r="AF1" s="28"/>
+      <c r="AG1" s="28"/>
+      <c r="AH1" s="28"/>
+      <c r="AI1" s="28"/>
+      <c r="AJ1" s="29"/>
+      <c r="AK1" s="27"/>
+      <c r="AL1" s="30"/>
+    </row>
+    <row r="2" s="23" customFormat="1" spans="1:38">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="33" t="s">
+      <c r="C2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="30"/>
-      <c r="O2" s="31"/>
-      <c r="P2" s="30"/>
-      <c r="Q2" s="30"/>
-      <c r="R2" s="30"/>
-      <c r="S2" s="30"/>
-      <c r="T2" s="30"/>
-      <c r="U2" s="30"/>
-      <c r="V2" s="30"/>
-      <c r="W2" s="30"/>
-      <c r="X2" s="30"/>
-      <c r="Y2" s="30"/>
-      <c r="Z2" s="30"/>
-      <c r="AA2" s="30"/>
-      <c r="AB2" s="30"/>
-      <c r="AC2" s="31"/>
-      <c r="AD2" s="31"/>
-      <c r="AE2" s="30"/>
-      <c r="AF2" s="30"/>
-      <c r="AG2" s="30"/>
-      <c r="AH2" s="30"/>
-      <c r="AI2" s="34"/>
-      <c r="AJ2" s="35" t="s">
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="28"/>
+      <c r="Q2" s="28"/>
+      <c r="R2" s="28"/>
+      <c r="S2" s="28"/>
+      <c r="T2" s="28"/>
+      <c r="U2" s="28"/>
+      <c r="V2" s="28"/>
+      <c r="W2" s="28"/>
+      <c r="X2" s="28"/>
+      <c r="Y2" s="28"/>
+      <c r="Z2" s="28"/>
+      <c r="AA2" s="28"/>
+      <c r="AB2" s="28"/>
+      <c r="AC2" s="29"/>
+      <c r="AD2" s="29"/>
+      <c r="AE2" s="28"/>
+      <c r="AF2" s="28"/>
+      <c r="AG2" s="28"/>
+      <c r="AH2" s="28"/>
+      <c r="AI2" s="32"/>
+      <c r="AJ2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="AK2" s="33" t="s">
+      <c r="AK2" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="AL2" s="33" t="s">
+      <c r="AL2" s="31" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" s="25" customFormat="1" ht="24" spans="1:38">
-      <c r="A3" s="36"/>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="38" t="s">
+    <row r="3" s="23" customFormat="1" ht="24" spans="1:38">
+      <c r="A3" s="34"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="38" t="s">
+      <c r="F3" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="38" t="s">
+      <c r="G3" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="38" t="s">
+      <c r="H3" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="38" t="s">
+      <c r="I3" s="36" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="38" t="s">
+      <c r="J3" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="38" t="s">
+      <c r="K3" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="38" t="s">
+      <c r="L3" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="M3" s="38" t="s">
+      <c r="M3" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="N3" s="38" t="s">
+      <c r="N3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="39" t="s">
+      <c r="O3" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="38" t="s">
+      <c r="P3" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="Q3" s="38" t="s">
+      <c r="Q3" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="38" t="s">
+      <c r="R3" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="S3" s="38" t="s">
+      <c r="S3" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="T3" s="38" t="s">
+      <c r="T3" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="U3" s="38" t="s">
+      <c r="U3" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="V3" s="38" t="s">
+      <c r="V3" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="W3" s="38" t="s">
+      <c r="W3" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="X3" s="38" t="s">
+      <c r="X3" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="Y3" s="38" t="s">
+      <c r="Y3" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="Z3" s="38" t="s">
+      <c r="Z3" s="36" t="s">
         <v>30</v>
       </c>
-      <c r="AA3" s="38" t="s">
+      <c r="AA3" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="AB3" s="38" t="s">
+      <c r="AB3" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="AC3" s="39" t="s">
+      <c r="AC3" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="AD3" s="39" t="s">
+      <c r="AD3" s="37" t="s">
         <v>34</v>
       </c>
-      <c r="AE3" s="38" t="s">
+      <c r="AE3" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="AF3" s="38" t="s">
+      <c r="AF3" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="AG3" s="38" t="s">
+      <c r="AG3" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="AH3" s="38" t="s">
+      <c r="AH3" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="AI3" s="38" t="s">
+      <c r="AI3" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="AJ3" s="40"/>
-      <c r="AK3" s="37"/>
-      <c r="AL3" s="37"/>
-    </row>
-    <row r="4" s="25" customFormat="1" spans="1:38">
-      <c r="A4" s="41">
+      <c r="AJ3" s="38"/>
+      <c r="AK3" s="35"/>
+      <c r="AL3" s="35"/>
+    </row>
+    <row r="4" s="23" customFormat="1" spans="1:38">
+      <c r="A4" s="39">
         <v>1</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="40" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="44" t="s">
+      <c r="D4" s="42" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="45">
+      <c r="E4" s="43">
         <v>9</v>
       </c>
-      <c r="F4" s="45">
+      <c r="F4" s="43">
         <v>9</v>
       </c>
-      <c r="G4" s="45">
+      <c r="G4" s="43">
         <v>9</v>
       </c>
-      <c r="H4" s="45">
+      <c r="H4" s="43">
         <v>9</v>
       </c>
-      <c r="I4" s="45">
+      <c r="I4" s="43">
         <v>9</v>
       </c>
-      <c r="J4" s="45">
+      <c r="J4" s="43">
         <v>9</v>
       </c>
-      <c r="K4" s="45">
+      <c r="K4" s="43">
         <v>9</v>
       </c>
-      <c r="L4" s="45">
+      <c r="L4" s="43">
         <v>9</v>
       </c>
-      <c r="M4" s="45">
+      <c r="M4" s="43">
         <v>9</v>
       </c>
-      <c r="N4" s="45">
+      <c r="N4" s="43">
         <v>9</v>
       </c>
-      <c r="O4" s="45">
+      <c r="O4" s="43">
         <v>9</v>
       </c>
-      <c r="P4" s="45">
+      <c r="P4" s="43">
         <v>9</v>
       </c>
-      <c r="Q4" s="45">
+      <c r="Q4" s="43">
         <v>9</v>
       </c>
-      <c r="R4" s="45">
+      <c r="R4" s="43">
         <v>9</v>
       </c>
-      <c r="S4" s="45">
+      <c r="S4" s="43">
         <v>9</v>
       </c>
-      <c r="T4" s="45">
+      <c r="T4" s="43">
         <v>9</v>
       </c>
-      <c r="U4" s="45">
+      <c r="U4" s="43">
         <v>9</v>
       </c>
-      <c r="V4" s="45">
+      <c r="V4" s="43">
         <v>9</v>
       </c>
-      <c r="W4" s="45">
+      <c r="W4" s="43">
         <v>9</v>
       </c>
-      <c r="X4" s="45">
+      <c r="X4" s="43">
         <v>9</v>
       </c>
-      <c r="Y4" s="45">
+      <c r="Y4" s="43">
         <v>9</v>
       </c>
-      <c r="Z4" s="45">
+      <c r="Z4" s="43">
         <v>9</v>
       </c>
-      <c r="AA4" s="45">
+      <c r="AA4" s="43">
         <v>9</v>
       </c>
-      <c r="AB4" s="45">
+      <c r="AB4" s="43">
         <v>9</v>
       </c>
-      <c r="AC4" s="45">
+      <c r="AC4" s="43">
         <v>9</v>
       </c>
-      <c r="AD4" s="45">
+      <c r="AD4" s="43">
         <v>9</v>
       </c>
-      <c r="AE4" s="45">
+      <c r="AE4" s="43">
         <v>9</v>
       </c>
-      <c r="AF4" s="45">
+      <c r="AF4" s="43">
         <v>9</v>
       </c>
-      <c r="AG4" s="45">
+      <c r="AG4" s="43">
         <v>9</v>
       </c>
-      <c r="AH4" s="45">
+      <c r="AH4" s="43">
         <v>9</v>
       </c>
-      <c r="AI4" s="45">
+      <c r="AI4" s="43">
         <v>4</v>
       </c>
-      <c r="AJ4" s="46">
+      <c r="AJ4" s="44">
         <f>SUM(E4:AI4)</f>
         <v>274</v>
       </c>
-      <c r="AK4" s="44">
+      <c r="AK4" s="42">
         <f>ROUND((AJ4+AJ5)/9,2)</f>
         <v>38</v>
       </c>
-      <c r="AL4" s="44" t="s">
+      <c r="AL4" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="5" s="25" customFormat="1" spans="1:38">
-      <c r="A5" s="41"/>
-      <c r="B5" s="80" t="s">
+    <row r="5" s="23" customFormat="1" spans="1:38">
+      <c r="A5" s="39"/>
+      <c r="B5" s="78" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="48"/>
-      <c r="D5" s="44" t="s">
+      <c r="C5" s="46"/>
+      <c r="D5" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45">
+      <c r="E5" s="43"/>
+      <c r="F5" s="43">
         <v>2</v>
       </c>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45">
+      <c r="G5" s="43"/>
+      <c r="H5" s="43">
         <v>3.5</v>
       </c>
-      <c r="I5" s="45">
+      <c r="I5" s="43">
         <v>3.5</v>
       </c>
-      <c r="J5" s="45">
+      <c r="J5" s="43">
         <v>2</v>
       </c>
-      <c r="K5" s="45">
+      <c r="K5" s="43">
         <v>3.5</v>
       </c>
-      <c r="L5" s="45">
+      <c r="L5" s="43">
         <v>3.5</v>
       </c>
-      <c r="M5" s="45">
+      <c r="M5" s="43">
         <v>3.5</v>
       </c>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45">
+      <c r="N5" s="43"/>
+      <c r="O5" s="43">
         <v>3.5</v>
       </c>
-      <c r="P5" s="45">
+      <c r="P5" s="43">
         <v>3.5</v>
       </c>
-      <c r="Q5" s="45">
+      <c r="Q5" s="43">
         <v>3.5</v>
       </c>
-      <c r="R5" s="45">
+      <c r="R5" s="43">
         <v>3.5</v>
       </c>
-      <c r="S5" s="45">
+      <c r="S5" s="43">
         <v>3.5</v>
       </c>
-      <c r="T5" s="45">
+      <c r="T5" s="43">
         <v>2</v>
       </c>
-      <c r="U5" s="45"/>
-      <c r="V5" s="45">
+      <c r="U5" s="43"/>
+      <c r="V5" s="43">
         <v>3.5</v>
       </c>
-      <c r="W5" s="45">
+      <c r="W5" s="43">
         <v>3.5</v>
       </c>
-      <c r="X5" s="45">
+      <c r="X5" s="43">
         <v>3.5</v>
       </c>
-      <c r="Y5" s="45"/>
-      <c r="Z5" s="45">
+      <c r="Y5" s="43"/>
+      <c r="Z5" s="43">
         <v>3</v>
       </c>
-      <c r="AA5" s="45">
+      <c r="AA5" s="43">
         <v>3</v>
       </c>
-      <c r="AB5" s="45"/>
-      <c r="AC5" s="45">
+      <c r="AB5" s="43"/>
+      <c r="AC5" s="43">
         <v>1.5</v>
       </c>
-      <c r="AD5" s="45">
+      <c r="AD5" s="43">
         <v>3</v>
       </c>
-      <c r="AE5" s="45">
+      <c r="AE5" s="43">
         <v>1.5</v>
       </c>
-      <c r="AF5" s="45">
+      <c r="AF5" s="43">
         <v>1.5</v>
       </c>
-      <c r="AG5" s="45">
+      <c r="AG5" s="43">
         <v>1.5</v>
       </c>
-      <c r="AH5" s="45">
+      <c r="AH5" s="43">
         <v>1.5</v>
       </c>
-      <c r="AI5" s="45"/>
-      <c r="AJ5" s="46">
+      <c r="AI5" s="43"/>
+      <c r="AJ5" s="44">
         <f>SUM(E5:AI5)</f>
         <v>68</v>
       </c>
-      <c r="AK5" s="44"/>
-      <c r="AL5" s="44"/>
-    </row>
-    <row r="6" s="25" customFormat="1" spans="1:38">
-      <c r="A6" s="41">
+      <c r="AK5" s="42"/>
+      <c r="AL5" s="42"/>
+    </row>
+    <row r="6" s="23" customFormat="1" spans="1:38">
+      <c r="A6" s="39">
         <v>2</v>
       </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="45"/>
-      <c r="M6" s="45"/>
-      <c r="N6" s="45"/>
-      <c r="O6" s="45"/>
-      <c r="P6" s="45"/>
-      <c r="Q6" s="45"/>
-      <c r="R6" s="45"/>
-      <c r="S6" s="45"/>
-      <c r="T6" s="45"/>
-      <c r="U6" s="45"/>
-      <c r="V6" s="45"/>
-      <c r="W6" s="45"/>
-      <c r="X6" s="45"/>
-      <c r="Y6" s="45"/>
-      <c r="Z6" s="45"/>
-      <c r="AA6" s="45"/>
-      <c r="AB6" s="45"/>
-      <c r="AC6" s="45"/>
-      <c r="AD6" s="45"/>
-      <c r="AE6" s="45"/>
-      <c r="AF6" s="45"/>
-      <c r="AG6" s="45"/>
-      <c r="AH6" s="45"/>
-      <c r="AI6" s="45"/>
-      <c r="AJ6" s="46"/>
-      <c r="AK6" s="44"/>
-      <c r="AL6" s="44" t="s">
+      <c r="B6" s="40"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="43"/>
+      <c r="L6" s="43"/>
+      <c r="M6" s="43"/>
+      <c r="N6" s="43"/>
+      <c r="O6" s="43"/>
+      <c r="P6" s="43"/>
+      <c r="Q6" s="43"/>
+      <c r="R6" s="43"/>
+      <c r="S6" s="43"/>
+      <c r="T6" s="43"/>
+      <c r="U6" s="43"/>
+      <c r="V6" s="43"/>
+      <c r="W6" s="43"/>
+      <c r="X6" s="43"/>
+      <c r="Y6" s="43"/>
+      <c r="Z6" s="43"/>
+      <c r="AA6" s="43"/>
+      <c r="AB6" s="43"/>
+      <c r="AC6" s="43"/>
+      <c r="AD6" s="43"/>
+      <c r="AE6" s="43"/>
+      <c r="AF6" s="43"/>
+      <c r="AG6" s="43"/>
+      <c r="AH6" s="43"/>
+      <c r="AI6" s="43"/>
+      <c r="AJ6" s="44"/>
+      <c r="AK6" s="42"/>
+      <c r="AL6" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="7" s="25" customFormat="1" spans="1:38">
-      <c r="A7" s="41"/>
-      <c r="B7" s="47"/>
-      <c r="C7" s="48"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
-      <c r="G7" s="45"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
-      <c r="K7" s="45"/>
-      <c r="L7" s="45"/>
-      <c r="M7" s="45"/>
-      <c r="N7" s="45"/>
-      <c r="O7" s="45"/>
-      <c r="P7" s="45"/>
-      <c r="Q7" s="45"/>
-      <c r="R7" s="45"/>
-      <c r="S7" s="45"/>
-      <c r="T7" s="45"/>
-      <c r="U7" s="45"/>
-      <c r="V7" s="45"/>
-      <c r="W7" s="45"/>
-      <c r="X7" s="45"/>
-      <c r="Y7" s="45"/>
-      <c r="Z7" s="45"/>
-      <c r="AA7" s="45"/>
-      <c r="AB7" s="45"/>
-      <c r="AC7" s="45"/>
-      <c r="AD7" s="45"/>
-      <c r="AE7" s="45"/>
-      <c r="AF7" s="45"/>
-      <c r="AG7" s="45"/>
-      <c r="AH7" s="45"/>
-      <c r="AI7" s="45"/>
-      <c r="AJ7" s="46"/>
-      <c r="AK7" s="44"/>
-      <c r="AL7" s="44"/>
-    </row>
-    <row r="8" s="25" customFormat="1" spans="1:38">
-      <c r="A8" s="41">
+    <row r="7" s="23" customFormat="1" spans="1:38">
+      <c r="A7" s="39"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="46"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
+      <c r="K7" s="43"/>
+      <c r="L7" s="43"/>
+      <c r="M7" s="43"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="43"/>
+      <c r="P7" s="43"/>
+      <c r="Q7" s="43"/>
+      <c r="R7" s="43"/>
+      <c r="S7" s="43"/>
+      <c r="T7" s="43"/>
+      <c r="U7" s="43"/>
+      <c r="V7" s="43"/>
+      <c r="W7" s="43"/>
+      <c r="X7" s="43"/>
+      <c r="Y7" s="43"/>
+      <c r="Z7" s="43"/>
+      <c r="AA7" s="43"/>
+      <c r="AB7" s="43"/>
+      <c r="AC7" s="43"/>
+      <c r="AD7" s="43"/>
+      <c r="AE7" s="43"/>
+      <c r="AF7" s="43"/>
+      <c r="AG7" s="43"/>
+      <c r="AH7" s="43"/>
+      <c r="AI7" s="43"/>
+      <c r="AJ7" s="44"/>
+      <c r="AK7" s="42"/>
+      <c r="AL7" s="42"/>
+    </row>
+    <row r="8" s="23" customFormat="1" spans="1:38">
+      <c r="A8" s="39">
         <v>3</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="44"/>
-      <c r="E8" s="45"/>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="45"/>
-      <c r="I8" s="45"/>
-      <c r="J8" s="45"/>
-      <c r="K8" s="45"/>
-      <c r="L8" s="45"/>
-      <c r="M8" s="45"/>
-      <c r="N8" s="45"/>
-      <c r="O8" s="45"/>
-      <c r="P8" s="45"/>
-      <c r="Q8" s="45"/>
-      <c r="R8" s="45"/>
-      <c r="S8" s="45"/>
-      <c r="T8" s="45"/>
-      <c r="U8" s="45"/>
-      <c r="V8" s="45"/>
-      <c r="W8" s="45"/>
-      <c r="X8" s="45"/>
-      <c r="Y8" s="45"/>
-      <c r="Z8" s="45"/>
-      <c r="AA8" s="45"/>
-      <c r="AB8" s="45"/>
-      <c r="AC8" s="45"/>
-      <c r="AD8" s="45"/>
-      <c r="AE8" s="45"/>
-      <c r="AF8" s="45"/>
-      <c r="AG8" s="45"/>
-      <c r="AH8" s="45"/>
-      <c r="AI8" s="45"/>
-      <c r="AJ8" s="46"/>
-      <c r="AK8" s="44"/>
-      <c r="AL8" s="44" t="s">
+      <c r="B8" s="40"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="42"/>
+      <c r="E8" s="43"/>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="43"/>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43"/>
+      <c r="K8" s="43"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="43"/>
+      <c r="N8" s="43"/>
+      <c r="O8" s="43"/>
+      <c r="P8" s="43"/>
+      <c r="Q8" s="43"/>
+      <c r="R8" s="43"/>
+      <c r="S8" s="43"/>
+      <c r="T8" s="43"/>
+      <c r="U8" s="43"/>
+      <c r="V8" s="43"/>
+      <c r="W8" s="43"/>
+      <c r="X8" s="43"/>
+      <c r="Y8" s="43"/>
+      <c r="Z8" s="43"/>
+      <c r="AA8" s="43"/>
+      <c r="AB8" s="43"/>
+      <c r="AC8" s="43"/>
+      <c r="AD8" s="43"/>
+      <c r="AE8" s="43"/>
+      <c r="AF8" s="43"/>
+      <c r="AG8" s="43"/>
+      <c r="AH8" s="43"/>
+      <c r="AI8" s="43"/>
+      <c r="AJ8" s="44"/>
+      <c r="AK8" s="42"/>
+      <c r="AL8" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="9" s="25" customFormat="1" spans="1:38">
-      <c r="A9" s="41"/>
-      <c r="B9" s="47"/>
-      <c r="C9" s="48"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="45"/>
-      <c r="J9" s="45"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="45"/>
-      <c r="M9" s="45"/>
-      <c r="N9" s="45"/>
-      <c r="O9" s="45"/>
-      <c r="P9" s="45"/>
-      <c r="Q9" s="45"/>
-      <c r="R9" s="45"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="45"/>
-      <c r="U9" s="45"/>
-      <c r="V9" s="45"/>
-      <c r="W9" s="45"/>
-      <c r="X9" s="45"/>
-      <c r="Y9" s="45"/>
-      <c r="Z9" s="45"/>
-      <c r="AA9" s="45"/>
-      <c r="AB9" s="45"/>
-      <c r="AC9" s="45"/>
-      <c r="AD9" s="45"/>
-      <c r="AE9" s="45"/>
-      <c r="AF9" s="45"/>
-      <c r="AG9" s="45"/>
-      <c r="AH9" s="45"/>
-      <c r="AI9" s="45"/>
-      <c r="AJ9" s="46"/>
-      <c r="AK9" s="44"/>
-      <c r="AL9" s="44"/>
-    </row>
-    <row r="10" s="25" customFormat="1" spans="1:38">
-      <c r="A10" s="41">
+    <row r="9" s="23" customFormat="1" spans="1:38">
+      <c r="A9" s="39"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="43"/>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+      <c r="H9" s="43"/>
+      <c r="I9" s="43"/>
+      <c r="J9" s="43"/>
+      <c r="K9" s="43"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="43"/>
+      <c r="N9" s="43"/>
+      <c r="O9" s="43"/>
+      <c r="P9" s="43"/>
+      <c r="Q9" s="43"/>
+      <c r="R9" s="43"/>
+      <c r="S9" s="43"/>
+      <c r="T9" s="43"/>
+      <c r="U9" s="43"/>
+      <c r="V9" s="43"/>
+      <c r="W9" s="43"/>
+      <c r="X9" s="43"/>
+      <c r="Y9" s="43"/>
+      <c r="Z9" s="43"/>
+      <c r="AA9" s="43"/>
+      <c r="AB9" s="43"/>
+      <c r="AC9" s="43"/>
+      <c r="AD9" s="43"/>
+      <c r="AE9" s="43"/>
+      <c r="AF9" s="43"/>
+      <c r="AG9" s="43"/>
+      <c r="AH9" s="43"/>
+      <c r="AI9" s="43"/>
+      <c r="AJ9" s="44"/>
+      <c r="AK9" s="42"/>
+      <c r="AL9" s="42"/>
+    </row>
+    <row r="10" s="23" customFormat="1" spans="1:38">
+      <c r="A10" s="39">
         <v>4</v>
       </c>
-      <c r="B10" s="42"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="45"/>
-      <c r="M10" s="45"/>
-      <c r="N10" s="45"/>
-      <c r="O10" s="45"/>
-      <c r="P10" s="45"/>
-      <c r="Q10" s="45"/>
-      <c r="R10" s="45"/>
-      <c r="S10" s="45"/>
-      <c r="T10" s="45"/>
-      <c r="U10" s="45"/>
-      <c r="V10" s="45"/>
-      <c r="W10" s="45"/>
-      <c r="X10" s="45"/>
-      <c r="Y10" s="45"/>
-      <c r="Z10" s="45"/>
-      <c r="AA10" s="45"/>
-      <c r="AB10" s="45"/>
-      <c r="AC10" s="45"/>
-      <c r="AD10" s="45"/>
-      <c r="AE10" s="45"/>
-      <c r="AF10" s="45"/>
-      <c r="AG10" s="45"/>
-      <c r="AH10" s="45"/>
-      <c r="AI10" s="45"/>
-      <c r="AJ10" s="46"/>
-      <c r="AK10" s="44"/>
-      <c r="AL10" s="44" t="s">
+      <c r="B10" s="40"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="43"/>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+      <c r="H10" s="43"/>
+      <c r="I10" s="43"/>
+      <c r="J10" s="43"/>
+      <c r="K10" s="43"/>
+      <c r="L10" s="43"/>
+      <c r="M10" s="43"/>
+      <c r="N10" s="43"/>
+      <c r="O10" s="43"/>
+      <c r="P10" s="43"/>
+      <c r="Q10" s="43"/>
+      <c r="R10" s="43"/>
+      <c r="S10" s="43"/>
+      <c r="T10" s="43"/>
+      <c r="U10" s="43"/>
+      <c r="V10" s="43"/>
+      <c r="W10" s="43"/>
+      <c r="X10" s="43"/>
+      <c r="Y10" s="43"/>
+      <c r="Z10" s="43"/>
+      <c r="AA10" s="43"/>
+      <c r="AB10" s="43"/>
+      <c r="AC10" s="43"/>
+      <c r="AD10" s="43"/>
+      <c r="AE10" s="43"/>
+      <c r="AF10" s="43"/>
+      <c r="AG10" s="43"/>
+      <c r="AH10" s="43"/>
+      <c r="AI10" s="43"/>
+      <c r="AJ10" s="44"/>
+      <c r="AK10" s="42"/>
+      <c r="AL10" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="11" s="25" customFormat="1" spans="1:38">
-      <c r="A11" s="41"/>
-      <c r="B11" s="47"/>
-      <c r="C11" s="48"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="45"/>
-      <c r="K11" s="45"/>
-      <c r="L11" s="45"/>
-      <c r="M11" s="45"/>
-      <c r="N11" s="45"/>
-      <c r="O11" s="45"/>
-      <c r="P11" s="45"/>
-      <c r="Q11" s="45"/>
-      <c r="R11" s="45"/>
-      <c r="S11" s="45"/>
-      <c r="T11" s="45"/>
-      <c r="U11" s="45"/>
-      <c r="V11" s="45"/>
-      <c r="W11" s="45"/>
-      <c r="X11" s="45"/>
-      <c r="Y11" s="45"/>
-      <c r="Z11" s="45"/>
-      <c r="AA11" s="45"/>
-      <c r="AB11" s="45"/>
-      <c r="AC11" s="45"/>
-      <c r="AD11" s="45"/>
-      <c r="AE11" s="45"/>
-      <c r="AF11" s="45"/>
-      <c r="AG11" s="45"/>
-      <c r="AH11" s="45"/>
-      <c r="AI11" s="45"/>
-      <c r="AJ11" s="46"/>
-      <c r="AK11" s="44"/>
-      <c r="AL11" s="44"/>
-    </row>
-    <row r="12" s="25" customFormat="1" spans="1:38">
-      <c r="A12" s="41">
+    <row r="11" s="23" customFormat="1" spans="1:38">
+      <c r="A11" s="39"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="43"/>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+      <c r="H11" s="43"/>
+      <c r="I11" s="43"/>
+      <c r="J11" s="43"/>
+      <c r="K11" s="43"/>
+      <c r="L11" s="43"/>
+      <c r="M11" s="43"/>
+      <c r="N11" s="43"/>
+      <c r="O11" s="43"/>
+      <c r="P11" s="43"/>
+      <c r="Q11" s="43"/>
+      <c r="R11" s="43"/>
+      <c r="S11" s="43"/>
+      <c r="T11" s="43"/>
+      <c r="U11" s="43"/>
+      <c r="V11" s="43"/>
+      <c r="W11" s="43"/>
+      <c r="X11" s="43"/>
+      <c r="Y11" s="43"/>
+      <c r="Z11" s="43"/>
+      <c r="AA11" s="43"/>
+      <c r="AB11" s="43"/>
+      <c r="AC11" s="43"/>
+      <c r="AD11" s="43"/>
+      <c r="AE11" s="43"/>
+      <c r="AF11" s="43"/>
+      <c r="AG11" s="43"/>
+      <c r="AH11" s="43"/>
+      <c r="AI11" s="43"/>
+      <c r="AJ11" s="44"/>
+      <c r="AK11" s="42"/>
+      <c r="AL11" s="42"/>
+    </row>
+    <row r="12" s="23" customFormat="1" spans="1:38">
+      <c r="A12" s="39">
         <v>5</v>
       </c>
-      <c r="B12" s="42"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
-      <c r="H12" s="45"/>
-      <c r="I12" s="45"/>
-      <c r="J12" s="45"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="45"/>
-      <c r="M12" s="45"/>
-      <c r="N12" s="45"/>
-      <c r="O12" s="45"/>
-      <c r="P12" s="45"/>
-      <c r="Q12" s="45"/>
-      <c r="R12" s="45"/>
-      <c r="S12" s="45"/>
-      <c r="T12" s="45"/>
-      <c r="U12" s="45"/>
-      <c r="V12" s="45"/>
-      <c r="W12" s="45"/>
-      <c r="X12" s="45"/>
-      <c r="Y12" s="45"/>
-      <c r="Z12" s="45"/>
-      <c r="AA12" s="45"/>
-      <c r="AB12" s="45"/>
-      <c r="AC12" s="45"/>
-      <c r="AD12" s="45"/>
-      <c r="AE12" s="45"/>
-      <c r="AF12" s="45"/>
-      <c r="AG12" s="45"/>
-      <c r="AH12" s="45"/>
-      <c r="AI12" s="45"/>
-      <c r="AJ12" s="46"/>
-      <c r="AK12" s="44"/>
-      <c r="AL12" s="44" t="s">
+      <c r="B12" s="40"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+      <c r="H12" s="43"/>
+      <c r="I12" s="43"/>
+      <c r="J12" s="43"/>
+      <c r="K12" s="43"/>
+      <c r="L12" s="43"/>
+      <c r="M12" s="43"/>
+      <c r="N12" s="43"/>
+      <c r="O12" s="43"/>
+      <c r="P12" s="43"/>
+      <c r="Q12" s="43"/>
+      <c r="R12" s="43"/>
+      <c r="S12" s="43"/>
+      <c r="T12" s="43"/>
+      <c r="U12" s="43"/>
+      <c r="V12" s="43"/>
+      <c r="W12" s="43"/>
+      <c r="X12" s="43"/>
+      <c r="Y12" s="43"/>
+      <c r="Z12" s="43"/>
+      <c r="AA12" s="43"/>
+      <c r="AB12" s="43"/>
+      <c r="AC12" s="43"/>
+      <c r="AD12" s="43"/>
+      <c r="AE12" s="43"/>
+      <c r="AF12" s="43"/>
+      <c r="AG12" s="43"/>
+      <c r="AH12" s="43"/>
+      <c r="AI12" s="43"/>
+      <c r="AJ12" s="44"/>
+      <c r="AK12" s="42"/>
+      <c r="AL12" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="13" s="25" customFormat="1" spans="1:38">
-      <c r="A13" s="41"/>
-      <c r="B13" s="47"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="45"/>
-      <c r="F13" s="45"/>
-      <c r="G13" s="45"/>
-      <c r="H13" s="45"/>
-      <c r="I13" s="45"/>
-      <c r="J13" s="45"/>
-      <c r="K13" s="45"/>
-      <c r="L13" s="45"/>
-      <c r="M13" s="45"/>
-      <c r="N13" s="45"/>
-      <c r="O13" s="45"/>
-      <c r="P13" s="45"/>
-      <c r="Q13" s="45"/>
-      <c r="R13" s="45"/>
-      <c r="S13" s="45"/>
-      <c r="T13" s="45"/>
-      <c r="U13" s="45"/>
-      <c r="V13" s="49"/>
-      <c r="W13" s="45"/>
-      <c r="X13" s="45"/>
-      <c r="Y13" s="45"/>
-      <c r="Z13" s="45"/>
-      <c r="AA13" s="45"/>
-      <c r="AB13" s="45"/>
-      <c r="AC13" s="45"/>
-      <c r="AD13" s="45"/>
-      <c r="AE13" s="45"/>
-      <c r="AF13" s="45"/>
-      <c r="AG13" s="45"/>
-      <c r="AH13" s="45"/>
-      <c r="AI13" s="45"/>
-      <c r="AJ13" s="46"/>
-      <c r="AK13" s="44"/>
-      <c r="AL13" s="44"/>
-    </row>
-    <row r="14" s="25" customFormat="1" spans="1:38">
-      <c r="A14" s="41">
+    <row r="13" s="23" customFormat="1" spans="1:38">
+      <c r="A13" s="39"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="46"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="43"/>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+      <c r="H13" s="43"/>
+      <c r="I13" s="43"/>
+      <c r="J13" s="43"/>
+      <c r="K13" s="43"/>
+      <c r="L13" s="43"/>
+      <c r="M13" s="43"/>
+      <c r="N13" s="43"/>
+      <c r="O13" s="43"/>
+      <c r="P13" s="43"/>
+      <c r="Q13" s="43"/>
+      <c r="R13" s="43"/>
+      <c r="S13" s="43"/>
+      <c r="T13" s="43"/>
+      <c r="U13" s="43"/>
+      <c r="V13" s="47"/>
+      <c r="W13" s="43"/>
+      <c r="X13" s="43"/>
+      <c r="Y13" s="43"/>
+      <c r="Z13" s="43"/>
+      <c r="AA13" s="43"/>
+      <c r="AB13" s="43"/>
+      <c r="AC13" s="43"/>
+      <c r="AD13" s="43"/>
+      <c r="AE13" s="43"/>
+      <c r="AF13" s="43"/>
+      <c r="AG13" s="43"/>
+      <c r="AH13" s="43"/>
+      <c r="AI13" s="43"/>
+      <c r="AJ13" s="44"/>
+      <c r="AK13" s="42"/>
+      <c r="AL13" s="42"/>
+    </row>
+    <row r="14" s="23" customFormat="1" spans="1:38">
+      <c r="A14" s="39">
         <v>6</v>
       </c>
-      <c r="B14" s="42"/>
-      <c r="C14" s="43"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="45"/>
-      <c r="L14" s="45"/>
-      <c r="M14" s="45"/>
-      <c r="N14" s="45"/>
-      <c r="O14" s="45"/>
-      <c r="P14" s="45"/>
-      <c r="Q14" s="45"/>
-      <c r="R14" s="45"/>
-      <c r="S14" s="45"/>
-      <c r="T14" s="45"/>
-      <c r="U14" s="45"/>
-      <c r="V14" s="45"/>
-      <c r="W14" s="45"/>
-      <c r="X14" s="45"/>
-      <c r="Y14" s="45"/>
-      <c r="Z14" s="45"/>
-      <c r="AA14" s="45"/>
-      <c r="AB14" s="45"/>
-      <c r="AC14" s="45"/>
-      <c r="AD14" s="45"/>
-      <c r="AE14" s="45"/>
-      <c r="AF14" s="45"/>
-      <c r="AG14" s="45"/>
-      <c r="AH14" s="45"/>
-      <c r="AI14" s="45"/>
-      <c r="AJ14" s="46"/>
-      <c r="AK14" s="44"/>
-      <c r="AL14" s="44" t="s">
+      <c r="B14" s="40"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="43"/>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+      <c r="H14" s="43"/>
+      <c r="I14" s="43"/>
+      <c r="J14" s="43"/>
+      <c r="K14" s="43"/>
+      <c r="L14" s="43"/>
+      <c r="M14" s="43"/>
+      <c r="N14" s="43"/>
+      <c r="O14" s="43"/>
+      <c r="P14" s="43"/>
+      <c r="Q14" s="43"/>
+      <c r="R14" s="43"/>
+      <c r="S14" s="43"/>
+      <c r="T14" s="43"/>
+      <c r="U14" s="43"/>
+      <c r="V14" s="43"/>
+      <c r="W14" s="43"/>
+      <c r="X14" s="43"/>
+      <c r="Y14" s="43"/>
+      <c r="Z14" s="43"/>
+      <c r="AA14" s="43"/>
+      <c r="AB14" s="43"/>
+      <c r="AC14" s="43"/>
+      <c r="AD14" s="43"/>
+      <c r="AE14" s="43"/>
+      <c r="AF14" s="43"/>
+      <c r="AG14" s="43"/>
+      <c r="AH14" s="43"/>
+      <c r="AI14" s="43"/>
+      <c r="AJ14" s="44"/>
+      <c r="AK14" s="42"/>
+      <c r="AL14" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="15" s="25" customFormat="1" spans="1:38">
-      <c r="A15" s="41"/>
-      <c r="B15" s="47"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="45"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45"/>
-      <c r="H15" s="45"/>
-      <c r="I15" s="45"/>
-      <c r="J15" s="45"/>
-      <c r="K15" s="45"/>
-      <c r="L15" s="45"/>
-      <c r="M15" s="45"/>
-      <c r="N15" s="45"/>
-      <c r="O15" s="45"/>
-      <c r="P15" s="45"/>
-      <c r="Q15" s="45"/>
-      <c r="R15" s="45"/>
-      <c r="S15" s="45"/>
-      <c r="T15" s="45"/>
-      <c r="U15" s="45"/>
-      <c r="V15" s="45"/>
-      <c r="W15" s="45"/>
-      <c r="X15" s="45"/>
-      <c r="Y15" s="45"/>
-      <c r="Z15" s="45"/>
-      <c r="AA15" s="45"/>
-      <c r="AB15" s="45"/>
-      <c r="AC15" s="45"/>
-      <c r="AD15" s="45"/>
-      <c r="AE15" s="45"/>
-      <c r="AF15" s="45"/>
-      <c r="AG15" s="45"/>
-      <c r="AH15" s="45"/>
-      <c r="AI15" s="45"/>
-      <c r="AJ15" s="46"/>
-      <c r="AK15" s="44"/>
-      <c r="AL15" s="44"/>
-    </row>
-    <row r="16" s="25" customFormat="1" spans="1:38">
-      <c r="A16" s="41">
+    <row r="15" s="23" customFormat="1" spans="1:38">
+      <c r="A15" s="39"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
+      <c r="H15" s="43"/>
+      <c r="I15" s="43"/>
+      <c r="J15" s="43"/>
+      <c r="K15" s="43"/>
+      <c r="L15" s="43"/>
+      <c r="M15" s="43"/>
+      <c r="N15" s="43"/>
+      <c r="O15" s="43"/>
+      <c r="P15" s="43"/>
+      <c r="Q15" s="43"/>
+      <c r="R15" s="43"/>
+      <c r="S15" s="43"/>
+      <c r="T15" s="43"/>
+      <c r="U15" s="43"/>
+      <c r="V15" s="43"/>
+      <c r="W15" s="43"/>
+      <c r="X15" s="43"/>
+      <c r="Y15" s="43"/>
+      <c r="Z15" s="43"/>
+      <c r="AA15" s="43"/>
+      <c r="AB15" s="43"/>
+      <c r="AC15" s="43"/>
+      <c r="AD15" s="43"/>
+      <c r="AE15" s="43"/>
+      <c r="AF15" s="43"/>
+      <c r="AG15" s="43"/>
+      <c r="AH15" s="43"/>
+      <c r="AI15" s="43"/>
+      <c r="AJ15" s="44"/>
+      <c r="AK15" s="42"/>
+      <c r="AL15" s="42"/>
+    </row>
+    <row r="16" s="23" customFormat="1" spans="1:38">
+      <c r="A16" s="39">
         <v>7</v>
       </c>
-      <c r="B16" s="50"/>
-      <c r="C16" s="43"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="45"/>
-      <c r="G16" s="45"/>
-      <c r="H16" s="45"/>
-      <c r="I16" s="45"/>
-      <c r="J16" s="45"/>
-      <c r="K16" s="45"/>
-      <c r="L16" s="45"/>
-      <c r="M16" s="45"/>
-      <c r="N16" s="45"/>
-      <c r="O16" s="45"/>
-      <c r="P16" s="45"/>
-      <c r="Q16" s="45"/>
-      <c r="R16" s="45"/>
-      <c r="S16" s="45"/>
-      <c r="T16" s="45"/>
-      <c r="U16" s="45"/>
-      <c r="V16" s="45"/>
-      <c r="W16" s="45"/>
-      <c r="X16" s="45"/>
-      <c r="Y16" s="45"/>
-      <c r="Z16" s="45"/>
-      <c r="AA16" s="45"/>
-      <c r="AB16" s="45"/>
-      <c r="AC16" s="45"/>
-      <c r="AD16" s="45"/>
-      <c r="AE16" s="45"/>
-      <c r="AF16" s="45"/>
-      <c r="AG16" s="45"/>
-      <c r="AH16" s="45"/>
-      <c r="AI16" s="45"/>
-      <c r="AJ16" s="46"/>
-      <c r="AK16" s="44"/>
-      <c r="AL16" s="44" t="s">
+      <c r="B16" s="48"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="42"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+      <c r="H16" s="43"/>
+      <c r="I16" s="43"/>
+      <c r="J16" s="43"/>
+      <c r="K16" s="43"/>
+      <c r="L16" s="43"/>
+      <c r="M16" s="43"/>
+      <c r="N16" s="43"/>
+      <c r="O16" s="43"/>
+      <c r="P16" s="43"/>
+      <c r="Q16" s="43"/>
+      <c r="R16" s="43"/>
+      <c r="S16" s="43"/>
+      <c r="T16" s="43"/>
+      <c r="U16" s="43"/>
+      <c r="V16" s="43"/>
+      <c r="W16" s="43"/>
+      <c r="X16" s="43"/>
+      <c r="Y16" s="43"/>
+      <c r="Z16" s="43"/>
+      <c r="AA16" s="43"/>
+      <c r="AB16" s="43"/>
+      <c r="AC16" s="43"/>
+      <c r="AD16" s="43"/>
+      <c r="AE16" s="43"/>
+      <c r="AF16" s="43"/>
+      <c r="AG16" s="43"/>
+      <c r="AH16" s="43"/>
+      <c r="AI16" s="43"/>
+      <c r="AJ16" s="44"/>
+      <c r="AK16" s="42"/>
+      <c r="AL16" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="17" s="25" customFormat="1" spans="1:38">
-      <c r="A17" s="41"/>
-      <c r="B17" s="51"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="45"/>
-      <c r="F17" s="45"/>
-      <c r="G17" s="45"/>
-      <c r="H17" s="45"/>
-      <c r="I17" s="45"/>
-      <c r="J17" s="45"/>
-      <c r="K17" s="45"/>
-      <c r="L17" s="45"/>
-      <c r="M17" s="45"/>
-      <c r="N17" s="45"/>
-      <c r="O17" s="45"/>
-      <c r="P17" s="45"/>
-      <c r="Q17" s="45"/>
-      <c r="R17" s="45"/>
-      <c r="S17" s="45"/>
-      <c r="T17" s="45"/>
-      <c r="U17" s="45"/>
-      <c r="V17" s="45"/>
-      <c r="W17" s="45"/>
-      <c r="X17" s="45"/>
-      <c r="Y17" s="45"/>
-      <c r="Z17" s="45"/>
-      <c r="AA17" s="45"/>
-      <c r="AB17" s="45"/>
-      <c r="AC17" s="45"/>
-      <c r="AD17" s="45"/>
-      <c r="AE17" s="45"/>
-      <c r="AF17" s="45"/>
-      <c r="AG17" s="45"/>
-      <c r="AH17" s="45"/>
-      <c r="AI17" s="45"/>
-      <c r="AJ17" s="46"/>
-      <c r="AK17" s="44"/>
-      <c r="AL17" s="44"/>
-    </row>
-    <row r="18" s="25" customFormat="1" spans="1:38">
-      <c r="A18" s="41">
+    <row r="17" s="23" customFormat="1" spans="1:38">
+      <c r="A17" s="39"/>
+      <c r="B17" s="49"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="42"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="43"/>
+      <c r="G17" s="43"/>
+      <c r="H17" s="43"/>
+      <c r="I17" s="43"/>
+      <c r="J17" s="43"/>
+      <c r="K17" s="43"/>
+      <c r="L17" s="43"/>
+      <c r="M17" s="43"/>
+      <c r="N17" s="43"/>
+      <c r="O17" s="43"/>
+      <c r="P17" s="43"/>
+      <c r="Q17" s="43"/>
+      <c r="R17" s="43"/>
+      <c r="S17" s="43"/>
+      <c r="T17" s="43"/>
+      <c r="U17" s="43"/>
+      <c r="V17" s="43"/>
+      <c r="W17" s="43"/>
+      <c r="X17" s="43"/>
+      <c r="Y17" s="43"/>
+      <c r="Z17" s="43"/>
+      <c r="AA17" s="43"/>
+      <c r="AB17" s="43"/>
+      <c r="AC17" s="43"/>
+      <c r="AD17" s="43"/>
+      <c r="AE17" s="43"/>
+      <c r="AF17" s="43"/>
+      <c r="AG17" s="43"/>
+      <c r="AH17" s="43"/>
+      <c r="AI17" s="43"/>
+      <c r="AJ17" s="44"/>
+      <c r="AK17" s="42"/>
+      <c r="AL17" s="42"/>
+    </row>
+    <row r="18" s="23" customFormat="1" spans="1:38">
+      <c r="A18" s="39">
         <v>8</v>
       </c>
-      <c r="B18" s="42"/>
-      <c r="C18" s="43"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="45"/>
-      <c r="J18" s="45"/>
-      <c r="K18" s="45"/>
-      <c r="L18" s="45"/>
-      <c r="M18" s="45"/>
-      <c r="N18" s="45"/>
-      <c r="O18" s="45"/>
-      <c r="P18" s="45"/>
-      <c r="Q18" s="45"/>
-      <c r="R18" s="45"/>
-      <c r="S18" s="45"/>
-      <c r="T18" s="45"/>
-      <c r="U18" s="45"/>
-      <c r="V18" s="45"/>
-      <c r="W18" s="45"/>
-      <c r="X18" s="45"/>
-      <c r="Y18" s="45"/>
-      <c r="Z18" s="45"/>
-      <c r="AA18" s="45"/>
-      <c r="AB18" s="45"/>
-      <c r="AC18" s="45"/>
-      <c r="AD18" s="45"/>
-      <c r="AE18" s="45"/>
-      <c r="AF18" s="45"/>
-      <c r="AG18" s="45"/>
-      <c r="AH18" s="45"/>
-      <c r="AI18" s="45"/>
-      <c r="AJ18" s="46"/>
-      <c r="AK18" s="44"/>
-      <c r="AL18" s="44" t="s">
+      <c r="B18" s="40"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+      <c r="H18" s="43"/>
+      <c r="I18" s="43"/>
+      <c r="J18" s="43"/>
+      <c r="K18" s="43"/>
+      <c r="L18" s="43"/>
+      <c r="M18" s="43"/>
+      <c r="N18" s="43"/>
+      <c r="O18" s="43"/>
+      <c r="P18" s="43"/>
+      <c r="Q18" s="43"/>
+      <c r="R18" s="43"/>
+      <c r="S18" s="43"/>
+      <c r="T18" s="43"/>
+      <c r="U18" s="43"/>
+      <c r="V18" s="43"/>
+      <c r="W18" s="43"/>
+      <c r="X18" s="43"/>
+      <c r="Y18" s="43"/>
+      <c r="Z18" s="43"/>
+      <c r="AA18" s="43"/>
+      <c r="AB18" s="43"/>
+      <c r="AC18" s="43"/>
+      <c r="AD18" s="43"/>
+      <c r="AE18" s="43"/>
+      <c r="AF18" s="43"/>
+      <c r="AG18" s="43"/>
+      <c r="AH18" s="43"/>
+      <c r="AI18" s="43"/>
+      <c r="AJ18" s="44"/>
+      <c r="AK18" s="42"/>
+      <c r="AL18" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="19" s="25" customFormat="1" spans="1:38">
-      <c r="A19" s="41"/>
-      <c r="B19" s="47"/>
-      <c r="C19" s="48"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="45"/>
-      <c r="F19" s="45"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="45"/>
-      <c r="I19" s="45"/>
-      <c r="J19" s="45"/>
-      <c r="K19" s="45"/>
-      <c r="L19" s="45"/>
-      <c r="M19" s="45"/>
-      <c r="N19" s="45"/>
-      <c r="O19" s="45"/>
-      <c r="P19" s="45"/>
-      <c r="Q19" s="45"/>
-      <c r="R19" s="45"/>
-      <c r="S19" s="45"/>
-      <c r="T19" s="45"/>
-      <c r="U19" s="45"/>
-      <c r="V19" s="45"/>
-      <c r="W19" s="45"/>
-      <c r="X19" s="45"/>
-      <c r="Y19" s="45"/>
-      <c r="Z19" s="45"/>
-      <c r="AA19" s="45"/>
-      <c r="AB19" s="45"/>
-      <c r="AC19" s="45"/>
-      <c r="AD19" s="45"/>
-      <c r="AE19" s="45"/>
-      <c r="AF19" s="45"/>
-      <c r="AG19" s="45"/>
-      <c r="AH19" s="45"/>
-      <c r="AI19" s="45"/>
-      <c r="AJ19" s="46"/>
-      <c r="AK19" s="44"/>
-      <c r="AL19" s="44"/>
-    </row>
-    <row r="20" s="25" customFormat="1" spans="1:38">
-      <c r="A20" s="41">
+    <row r="19" s="23" customFormat="1" spans="1:38">
+      <c r="A19" s="39"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="43"/>
+      <c r="I19" s="43"/>
+      <c r="J19" s="43"/>
+      <c r="K19" s="43"/>
+      <c r="L19" s="43"/>
+      <c r="M19" s="43"/>
+      <c r="N19" s="43"/>
+      <c r="O19" s="43"/>
+      <c r="P19" s="43"/>
+      <c r="Q19" s="43"/>
+      <c r="R19" s="43"/>
+      <c r="S19" s="43"/>
+      <c r="T19" s="43"/>
+      <c r="U19" s="43"/>
+      <c r="V19" s="43"/>
+      <c r="W19" s="43"/>
+      <c r="X19" s="43"/>
+      <c r="Y19" s="43"/>
+      <c r="Z19" s="43"/>
+      <c r="AA19" s="43"/>
+      <c r="AB19" s="43"/>
+      <c r="AC19" s="43"/>
+      <c r="AD19" s="43"/>
+      <c r="AE19" s="43"/>
+      <c r="AF19" s="43"/>
+      <c r="AG19" s="43"/>
+      <c r="AH19" s="43"/>
+      <c r="AI19" s="43"/>
+      <c r="AJ19" s="44"/>
+      <c r="AK19" s="42"/>
+      <c r="AL19" s="42"/>
+    </row>
+    <row r="20" s="23" customFormat="1" spans="1:38">
+      <c r="A20" s="39">
         <v>9</v>
       </c>
-      <c r="B20" s="50"/>
-      <c r="C20" s="43"/>
-      <c r="D20" s="44"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="45"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="45"/>
-      <c r="J20" s="45"/>
-      <c r="K20" s="45"/>
-      <c r="L20" s="45"/>
-      <c r="M20" s="45"/>
-      <c r="N20" s="45"/>
-      <c r="O20" s="45"/>
-      <c r="P20" s="45"/>
-      <c r="Q20" s="45"/>
-      <c r="R20" s="45"/>
-      <c r="S20" s="45"/>
-      <c r="T20" s="45"/>
-      <c r="U20" s="45"/>
-      <c r="V20" s="45"/>
-      <c r="W20" s="45"/>
-      <c r="X20" s="45"/>
-      <c r="Y20" s="45"/>
-      <c r="Z20" s="45"/>
-      <c r="AA20" s="45"/>
-      <c r="AB20" s="45"/>
-      <c r="AC20" s="45"/>
-      <c r="AD20" s="45"/>
-      <c r="AE20" s="45"/>
-      <c r="AF20" s="45"/>
-      <c r="AG20" s="45"/>
-      <c r="AH20" s="45"/>
-      <c r="AI20" s="45"/>
-      <c r="AJ20" s="46"/>
-      <c r="AK20" s="44"/>
-      <c r="AL20" s="44" t="s">
+      <c r="B20" s="48"/>
+      <c r="C20" s="41"/>
+      <c r="D20" s="42"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="43"/>
+      <c r="G20" s="43"/>
+      <c r="H20" s="43"/>
+      <c r="I20" s="43"/>
+      <c r="J20" s="43"/>
+      <c r="K20" s="43"/>
+      <c r="L20" s="43"/>
+      <c r="M20" s="43"/>
+      <c r="N20" s="43"/>
+      <c r="O20" s="43"/>
+      <c r="P20" s="43"/>
+      <c r="Q20" s="43"/>
+      <c r="R20" s="43"/>
+      <c r="S20" s="43"/>
+      <c r="T20" s="43"/>
+      <c r="U20" s="43"/>
+      <c r="V20" s="43"/>
+      <c r="W20" s="43"/>
+      <c r="X20" s="43"/>
+      <c r="Y20" s="43"/>
+      <c r="Z20" s="43"/>
+      <c r="AA20" s="43"/>
+      <c r="AB20" s="43"/>
+      <c r="AC20" s="43"/>
+      <c r="AD20" s="43"/>
+      <c r="AE20" s="43"/>
+      <c r="AF20" s="43"/>
+      <c r="AG20" s="43"/>
+      <c r="AH20" s="43"/>
+      <c r="AI20" s="43"/>
+      <c r="AJ20" s="44"/>
+      <c r="AK20" s="42"/>
+      <c r="AL20" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="21" s="25" customFormat="1" spans="1:38">
-      <c r="A21" s="41"/>
-      <c r="B21" s="51"/>
-      <c r="C21" s="48"/>
-      <c r="D21" s="44"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="45"/>
-      <c r="G21" s="45"/>
-      <c r="H21" s="45"/>
-      <c r="I21" s="45"/>
-      <c r="J21" s="45"/>
-      <c r="K21" s="45"/>
-      <c r="L21" s="45"/>
-      <c r="M21" s="45"/>
-      <c r="N21" s="45"/>
-      <c r="O21" s="45"/>
-      <c r="P21" s="45"/>
-      <c r="Q21" s="45"/>
-      <c r="R21" s="45"/>
-      <c r="S21" s="45"/>
-      <c r="T21" s="45"/>
-      <c r="U21" s="45"/>
-      <c r="V21" s="45"/>
-      <c r="W21" s="45"/>
-      <c r="X21" s="45"/>
-      <c r="Y21" s="45"/>
-      <c r="Z21" s="45"/>
-      <c r="AA21" s="45"/>
-      <c r="AB21" s="45"/>
-      <c r="AC21" s="45"/>
-      <c r="AD21" s="45"/>
-      <c r="AE21" s="45"/>
-      <c r="AF21" s="45"/>
-      <c r="AG21" s="45"/>
-      <c r="AH21" s="45"/>
-      <c r="AI21" s="45"/>
-      <c r="AJ21" s="46"/>
-      <c r="AK21" s="44"/>
-      <c r="AL21" s="44"/>
-    </row>
-    <row r="22" s="25" customFormat="1" spans="1:38">
-      <c r="A22" s="41">
+    <row r="21" s="23" customFormat="1" spans="1:38">
+      <c r="A21" s="39"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="46"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+      <c r="H21" s="43"/>
+      <c r="I21" s="43"/>
+      <c r="J21" s="43"/>
+      <c r="K21" s="43"/>
+      <c r="L21" s="43"/>
+      <c r="M21" s="43"/>
+      <c r="N21" s="43"/>
+      <c r="O21" s="43"/>
+      <c r="P21" s="43"/>
+      <c r="Q21" s="43"/>
+      <c r="R21" s="43"/>
+      <c r="S21" s="43"/>
+      <c r="T21" s="43"/>
+      <c r="U21" s="43"/>
+      <c r="V21" s="43"/>
+      <c r="W21" s="43"/>
+      <c r="X21" s="43"/>
+      <c r="Y21" s="43"/>
+      <c r="Z21" s="43"/>
+      <c r="AA21" s="43"/>
+      <c r="AB21" s="43"/>
+      <c r="AC21" s="43"/>
+      <c r="AD21" s="43"/>
+      <c r="AE21" s="43"/>
+      <c r="AF21" s="43"/>
+      <c r="AG21" s="43"/>
+      <c r="AH21" s="43"/>
+      <c r="AI21" s="43"/>
+      <c r="AJ21" s="44"/>
+      <c r="AK21" s="42"/>
+      <c r="AL21" s="42"/>
+    </row>
+    <row r="22" s="23" customFormat="1" spans="1:38">
+      <c r="A22" s="39">
         <v>10</v>
       </c>
-      <c r="B22" s="50"/>
-      <c r="C22" s="43"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="45"/>
-      <c r="J22" s="45"/>
-      <c r="K22" s="45"/>
-      <c r="L22" s="45"/>
-      <c r="M22" s="45"/>
-      <c r="N22" s="45"/>
-      <c r="O22" s="45"/>
-      <c r="P22" s="45"/>
-      <c r="Q22" s="45"/>
-      <c r="R22" s="45"/>
-      <c r="S22" s="45"/>
-      <c r="T22" s="45"/>
-      <c r="U22" s="45"/>
-      <c r="V22" s="45"/>
-      <c r="W22" s="45"/>
-      <c r="X22" s="45"/>
-      <c r="Y22" s="45"/>
-      <c r="Z22" s="45"/>
-      <c r="AA22" s="45"/>
-      <c r="AB22" s="45"/>
-      <c r="AC22" s="45"/>
-      <c r="AD22" s="45"/>
-      <c r="AE22" s="45"/>
-      <c r="AF22" s="45"/>
-      <c r="AG22" s="45"/>
-      <c r="AH22" s="45"/>
-      <c r="AI22" s="45"/>
-      <c r="AJ22" s="46"/>
-      <c r="AK22" s="44"/>
-      <c r="AL22" s="44" t="s">
+      <c r="B22" s="48"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="43"/>
+      <c r="J22" s="43"/>
+      <c r="K22" s="43"/>
+      <c r="L22" s="43"/>
+      <c r="M22" s="43"/>
+      <c r="N22" s="43"/>
+      <c r="O22" s="43"/>
+      <c r="P22" s="43"/>
+      <c r="Q22" s="43"/>
+      <c r="R22" s="43"/>
+      <c r="S22" s="43"/>
+      <c r="T22" s="43"/>
+      <c r="U22" s="43"/>
+      <c r="V22" s="43"/>
+      <c r="W22" s="43"/>
+      <c r="X22" s="43"/>
+      <c r="Y22" s="43"/>
+      <c r="Z22" s="43"/>
+      <c r="AA22" s="43"/>
+      <c r="AB22" s="43"/>
+      <c r="AC22" s="43"/>
+      <c r="AD22" s="43"/>
+      <c r="AE22" s="43"/>
+      <c r="AF22" s="43"/>
+      <c r="AG22" s="43"/>
+      <c r="AH22" s="43"/>
+      <c r="AI22" s="43"/>
+      <c r="AJ22" s="44"/>
+      <c r="AK22" s="42"/>
+      <c r="AL22" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" s="25" customFormat="1" spans="1:38">
-      <c r="A23" s="41"/>
-      <c r="B23" s="51"/>
-      <c r="C23" s="48"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="45"/>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="45"/>
-      <c r="I23" s="45"/>
-      <c r="J23" s="45"/>
-      <c r="K23" s="45"/>
-      <c r="L23" s="45"/>
-      <c r="M23" s="45"/>
-      <c r="N23" s="45"/>
-      <c r="O23" s="45"/>
-      <c r="P23" s="45"/>
-      <c r="Q23" s="45"/>
-      <c r="R23" s="45"/>
-      <c r="S23" s="45"/>
-      <c r="T23" s="45"/>
-      <c r="U23" s="45"/>
-      <c r="V23" s="45"/>
-      <c r="W23" s="45"/>
-      <c r="X23" s="45"/>
-      <c r="Y23" s="45"/>
-      <c r="Z23" s="45"/>
-      <c r="AA23" s="45"/>
-      <c r="AB23" s="45"/>
-      <c r="AC23" s="45"/>
-      <c r="AD23" s="45"/>
-      <c r="AE23" s="45"/>
-      <c r="AF23" s="45"/>
-      <c r="AG23" s="45"/>
-      <c r="AH23" s="45"/>
-      <c r="AI23" s="45"/>
-      <c r="AJ23" s="46"/>
-      <c r="AK23" s="44"/>
-      <c r="AL23" s="44"/>
-    </row>
-    <row r="24" s="25" customFormat="1" spans="1:38">
-      <c r="A24" s="41">
+    <row r="23" s="23" customFormat="1" spans="1:38">
+      <c r="A23" s="39"/>
+      <c r="B23" s="49"/>
+      <c r="C23" s="46"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+      <c r="H23" s="43"/>
+      <c r="I23" s="43"/>
+      <c r="J23" s="43"/>
+      <c r="K23" s="43"/>
+      <c r="L23" s="43"/>
+      <c r="M23" s="43"/>
+      <c r="N23" s="43"/>
+      <c r="O23" s="43"/>
+      <c r="P23" s="43"/>
+      <c r="Q23" s="43"/>
+      <c r="R23" s="43"/>
+      <c r="S23" s="43"/>
+      <c r="T23" s="43"/>
+      <c r="U23" s="43"/>
+      <c r="V23" s="43"/>
+      <c r="W23" s="43"/>
+      <c r="X23" s="43"/>
+      <c r="Y23" s="43"/>
+      <c r="Z23" s="43"/>
+      <c r="AA23" s="43"/>
+      <c r="AB23" s="43"/>
+      <c r="AC23" s="43"/>
+      <c r="AD23" s="43"/>
+      <c r="AE23" s="43"/>
+      <c r="AF23" s="43"/>
+      <c r="AG23" s="43"/>
+      <c r="AH23" s="43"/>
+      <c r="AI23" s="43"/>
+      <c r="AJ23" s="44"/>
+      <c r="AK23" s="42"/>
+      <c r="AL23" s="42"/>
+    </row>
+    <row r="24" s="23" customFormat="1" spans="1:38">
+      <c r="A24" s="39">
         <v>11</v>
       </c>
-      <c r="B24" s="50"/>
-      <c r="C24" s="43"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
-      <c r="H24" s="45"/>
-      <c r="I24" s="45"/>
-      <c r="J24" s="45"/>
-      <c r="K24" s="45"/>
-      <c r="L24" s="45"/>
-      <c r="M24" s="45"/>
-      <c r="N24" s="45"/>
-      <c r="O24" s="45"/>
-      <c r="P24" s="45"/>
-      <c r="Q24" s="45"/>
-      <c r="R24" s="45"/>
-      <c r="S24" s="45"/>
-      <c r="T24" s="45"/>
-      <c r="U24" s="45"/>
-      <c r="V24" s="45"/>
-      <c r="W24" s="45"/>
-      <c r="X24" s="45"/>
-      <c r="Y24" s="45"/>
-      <c r="Z24" s="45"/>
-      <c r="AA24" s="45"/>
-      <c r="AB24" s="52"/>
-      <c r="AC24" s="45"/>
-      <c r="AD24" s="45"/>
-      <c r="AE24" s="45"/>
-      <c r="AF24" s="45"/>
-      <c r="AG24" s="45"/>
-      <c r="AH24" s="45"/>
-      <c r="AI24" s="45"/>
-      <c r="AJ24" s="46"/>
-      <c r="AK24" s="44"/>
-      <c r="AL24" s="44" t="s">
+      <c r="B24" s="48"/>
+      <c r="C24" s="41"/>
+      <c r="D24" s="42"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="43"/>
+      <c r="H24" s="43"/>
+      <c r="I24" s="43"/>
+      <c r="J24" s="43"/>
+      <c r="K24" s="43"/>
+      <c r="L24" s="43"/>
+      <c r="M24" s="43"/>
+      <c r="N24" s="43"/>
+      <c r="O24" s="43"/>
+      <c r="P24" s="43"/>
+      <c r="Q24" s="43"/>
+      <c r="R24" s="43"/>
+      <c r="S24" s="43"/>
+      <c r="T24" s="43"/>
+      <c r="U24" s="43"/>
+      <c r="V24" s="43"/>
+      <c r="W24" s="43"/>
+      <c r="X24" s="43"/>
+      <c r="Y24" s="43"/>
+      <c r="Z24" s="43"/>
+      <c r="AA24" s="43"/>
+      <c r="AB24" s="50"/>
+      <c r="AC24" s="43"/>
+      <c r="AD24" s="43"/>
+      <c r="AE24" s="43"/>
+      <c r="AF24" s="43"/>
+      <c r="AG24" s="43"/>
+      <c r="AH24" s="43"/>
+      <c r="AI24" s="43"/>
+      <c r="AJ24" s="44"/>
+      <c r="AK24" s="42"/>
+      <c r="AL24" s="42" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="25" s="25" customFormat="1" spans="1:38">
-      <c r="A25" s="53"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="54"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="54"/>
-      <c r="H25" s="54"/>
-      <c r="I25" s="54"/>
-      <c r="J25" s="54"/>
-      <c r="K25" s="54"/>
-      <c r="L25" s="54"/>
-      <c r="M25" s="54"/>
-      <c r="N25" s="54"/>
-      <c r="O25" s="54"/>
-      <c r="P25" s="54"/>
-      <c r="Q25" s="54"/>
-      <c r="R25" s="54"/>
-      <c r="S25" s="54"/>
-      <c r="T25" s="54"/>
-      <c r="U25" s="54"/>
-      <c r="V25" s="54"/>
-      <c r="W25" s="54"/>
-      <c r="X25" s="54"/>
-      <c r="Y25" s="54"/>
-      <c r="Z25" s="54"/>
-      <c r="AA25" s="54"/>
-      <c r="AB25" s="54"/>
-      <c r="AC25" s="54"/>
-      <c r="AD25" s="54"/>
-      <c r="AE25" s="54"/>
-      <c r="AF25" s="54"/>
-      <c r="AG25" s="54"/>
-      <c r="AH25" s="54"/>
-      <c r="AI25" s="54"/>
-      <c r="AJ25" s="55"/>
-      <c r="AK25" s="43"/>
-      <c r="AL25" s="43"/>
-    </row>
-    <row r="26" s="25" customFormat="1" spans="1:38">
-      <c r="A26" s="56">
+    <row r="25" s="23" customFormat="1" spans="1:38">
+      <c r="A25" s="51"/>
+      <c r="B25" s="49"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="41"/>
+      <c r="E25" s="52"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="52"/>
+      <c r="H25" s="52"/>
+      <c r="I25" s="52"/>
+      <c r="J25" s="52"/>
+      <c r="K25" s="52"/>
+      <c r="L25" s="52"/>
+      <c r="M25" s="52"/>
+      <c r="N25" s="52"/>
+      <c r="O25" s="52"/>
+      <c r="P25" s="52"/>
+      <c r="Q25" s="52"/>
+      <c r="R25" s="52"/>
+      <c r="S25" s="52"/>
+      <c r="T25" s="52"/>
+      <c r="U25" s="52"/>
+      <c r="V25" s="52"/>
+      <c r="W25" s="52"/>
+      <c r="X25" s="52"/>
+      <c r="Y25" s="52"/>
+      <c r="Z25" s="52"/>
+      <c r="AA25" s="52"/>
+      <c r="AB25" s="52"/>
+      <c r="AC25" s="52"/>
+      <c r="AD25" s="52"/>
+      <c r="AE25" s="52"/>
+      <c r="AF25" s="52"/>
+      <c r="AG25" s="52"/>
+      <c r="AH25" s="52"/>
+      <c r="AI25" s="52"/>
+      <c r="AJ25" s="53"/>
+      <c r="AK25" s="41"/>
+      <c r="AL25" s="41"/>
+    </row>
+    <row r="26" s="23" customFormat="1" spans="1:38">
+      <c r="A26" s="54">
         <v>12</v>
       </c>
-      <c r="B26" s="50"/>
-      <c r="C26" s="43"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="57"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="57"/>
-      <c r="K26" s="57"/>
-      <c r="L26" s="57"/>
-      <c r="M26" s="57"/>
-      <c r="N26" s="57"/>
-      <c r="O26" s="45"/>
-      <c r="P26" s="57"/>
-      <c r="Q26" s="57"/>
-      <c r="R26" s="57"/>
-      <c r="S26" s="57"/>
-      <c r="T26" s="57"/>
-      <c r="U26" s="57"/>
-      <c r="V26" s="57"/>
-      <c r="W26" s="57"/>
-      <c r="X26" s="57"/>
-      <c r="Y26" s="57"/>
-      <c r="Z26" s="57"/>
-      <c r="AA26" s="57"/>
-      <c r="AB26" s="57"/>
-      <c r="AC26" s="45"/>
-      <c r="AD26" s="45"/>
-      <c r="AE26" s="57"/>
-      <c r="AF26" s="57"/>
-      <c r="AG26" s="57"/>
-      <c r="AH26" s="57"/>
-      <c r="AI26" s="57"/>
-      <c r="AJ26" s="46"/>
-      <c r="AK26" s="44"/>
-      <c r="AL26" s="58"/>
-    </row>
-    <row r="27" s="25" customFormat="1" spans="1:38">
-      <c r="A27" s="56"/>
-      <c r="B27" s="51"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="59"/>
-      <c r="F27" s="54"/>
-      <c r="G27" s="57"/>
-      <c r="H27" s="54"/>
-      <c r="I27" s="54"/>
-      <c r="J27" s="54"/>
-      <c r="K27" s="54"/>
-      <c r="L27" s="54"/>
-      <c r="M27" s="54"/>
-      <c r="N27" s="54"/>
-      <c r="O27" s="54"/>
-      <c r="P27" s="54"/>
-      <c r="Q27" s="54"/>
-      <c r="R27" s="54"/>
-      <c r="S27" s="45"/>
-      <c r="T27" s="45"/>
-      <c r="U27" s="45"/>
-      <c r="V27" s="54"/>
-      <c r="W27" s="54"/>
-      <c r="X27" s="54"/>
-      <c r="Y27" s="45"/>
-      <c r="Z27" s="45"/>
-      <c r="AA27" s="45"/>
-      <c r="AB27" s="45"/>
-      <c r="AC27" s="60"/>
-      <c r="AD27" s="60"/>
-      <c r="AE27" s="54"/>
-      <c r="AF27" s="54"/>
-      <c r="AG27" s="54"/>
-      <c r="AH27" s="54"/>
-      <c r="AI27" s="59"/>
-      <c r="AJ27" s="55"/>
-      <c r="AK27" s="43"/>
-      <c r="AL27" s="61"/>
-    </row>
-    <row r="28" s="25" customFormat="1" spans="1:38">
-      <c r="A28" s="56">
+      <c r="B26" s="48"/>
+      <c r="C26" s="41"/>
+      <c r="D26" s="42"/>
+      <c r="E26" s="55"/>
+      <c r="F26" s="43"/>
+      <c r="G26" s="55"/>
+      <c r="H26" s="55"/>
+      <c r="I26" s="55"/>
+      <c r="J26" s="55"/>
+      <c r="K26" s="55"/>
+      <c r="L26" s="55"/>
+      <c r="M26" s="55"/>
+      <c r="N26" s="55"/>
+      <c r="O26" s="43"/>
+      <c r="P26" s="55"/>
+      <c r="Q26" s="55"/>
+      <c r="R26" s="55"/>
+      <c r="S26" s="55"/>
+      <c r="T26" s="55"/>
+      <c r="U26" s="55"/>
+      <c r="V26" s="55"/>
+      <c r="W26" s="55"/>
+      <c r="X26" s="55"/>
+      <c r="Y26" s="55"/>
+      <c r="Z26" s="55"/>
+      <c r="AA26" s="55"/>
+      <c r="AB26" s="55"/>
+      <c r="AC26" s="43"/>
+      <c r="AD26" s="43"/>
+      <c r="AE26" s="55"/>
+      <c r="AF26" s="55"/>
+      <c r="AG26" s="55"/>
+      <c r="AH26" s="55"/>
+      <c r="AI26" s="55"/>
+      <c r="AJ26" s="44"/>
+      <c r="AK26" s="42"/>
+      <c r="AL26" s="56"/>
+    </row>
+    <row r="27" s="23" customFormat="1" spans="1:38">
+      <c r="A27" s="54"/>
+      <c r="B27" s="49"/>
+      <c r="C27" s="46"/>
+      <c r="D27" s="41"/>
+      <c r="E27" s="57"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="52"/>
+      <c r="I27" s="52"/>
+      <c r="J27" s="52"/>
+      <c r="K27" s="52"/>
+      <c r="L27" s="52"/>
+      <c r="M27" s="52"/>
+      <c r="N27" s="52"/>
+      <c r="O27" s="52"/>
+      <c r="P27" s="52"/>
+      <c r="Q27" s="52"/>
+      <c r="R27" s="52"/>
+      <c r="S27" s="43"/>
+      <c r="T27" s="43"/>
+      <c r="U27" s="43"/>
+      <c r="V27" s="52"/>
+      <c r="W27" s="52"/>
+      <c r="X27" s="52"/>
+      <c r="Y27" s="43"/>
+      <c r="Z27" s="43"/>
+      <c r="AA27" s="43"/>
+      <c r="AB27" s="43"/>
+      <c r="AC27" s="58"/>
+      <c r="AD27" s="58"/>
+      <c r="AE27" s="52"/>
+      <c r="AF27" s="52"/>
+      <c r="AG27" s="52"/>
+      <c r="AH27" s="52"/>
+      <c r="AI27" s="57"/>
+      <c r="AJ27" s="53"/>
+      <c r="AK27" s="41"/>
+      <c r="AL27" s="59"/>
+    </row>
+    <row r="28" s="23" customFormat="1" spans="1:38">
+      <c r="A28" s="54">
         <v>13</v>
       </c>
-      <c r="B28" s="42"/>
-      <c r="C28" s="43"/>
-      <c r="D28" s="44"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="45"/>
-      <c r="G28" s="57"/>
-      <c r="H28" s="57"/>
-      <c r="I28" s="57"/>
-      <c r="J28" s="57"/>
-      <c r="K28" s="57"/>
-      <c r="L28" s="57"/>
-      <c r="M28" s="57"/>
-      <c r="N28" s="57"/>
-      <c r="O28" s="45"/>
-      <c r="P28" s="57"/>
-      <c r="Q28" s="57"/>
-      <c r="R28" s="57"/>
-      <c r="S28" s="57"/>
-      <c r="T28" s="57"/>
-      <c r="U28" s="57"/>
-      <c r="V28" s="57"/>
-      <c r="W28" s="57"/>
-      <c r="X28" s="57"/>
-      <c r="Y28" s="57"/>
-      <c r="Z28" s="57"/>
-      <c r="AA28" s="57"/>
-      <c r="AB28" s="57"/>
-      <c r="AC28" s="45"/>
-      <c r="AD28" s="45"/>
-      <c r="AE28" s="57"/>
-      <c r="AF28" s="57"/>
-      <c r="AG28" s="57"/>
-      <c r="AH28" s="57"/>
-      <c r="AI28" s="57"/>
-      <c r="AJ28" s="46"/>
-      <c r="AK28" s="44"/>
-      <c r="AL28" s="58"/>
-    </row>
-    <row r="29" s="25" customFormat="1" spans="1:38">
-      <c r="A29" s="62"/>
-      <c r="B29" s="47"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="63"/>
-      <c r="F29" s="54"/>
-      <c r="G29" s="64"/>
-      <c r="H29" s="54"/>
-      <c r="I29" s="54"/>
-      <c r="J29" s="54"/>
-      <c r="K29" s="54"/>
-      <c r="L29" s="54"/>
-      <c r="M29" s="54"/>
-      <c r="N29" s="54"/>
-      <c r="O29" s="54"/>
-      <c r="P29" s="54"/>
-      <c r="Q29" s="54"/>
-      <c r="R29" s="54"/>
-      <c r="S29" s="45"/>
-      <c r="T29" s="54"/>
-      <c r="U29" s="54"/>
-      <c r="V29" s="65"/>
-      <c r="W29" s="54"/>
-      <c r="X29" s="54"/>
-      <c r="Y29" s="54"/>
-      <c r="Z29" s="54"/>
-      <c r="AA29" s="54"/>
-      <c r="AB29" s="54"/>
-      <c r="AC29" s="66"/>
-      <c r="AD29" s="66"/>
-      <c r="AE29" s="54"/>
-      <c r="AF29" s="54"/>
-      <c r="AG29" s="54"/>
-      <c r="AH29" s="54"/>
-      <c r="AI29" s="64"/>
-      <c r="AJ29" s="55"/>
-      <c r="AK29" s="43"/>
-      <c r="AL29" s="67"/>
-    </row>
-    <row r="30" s="25" customFormat="1" spans="1:38">
-      <c r="A30" s="68" t="s">
+      <c r="B28" s="40"/>
+      <c r="C28" s="41"/>
+      <c r="D28" s="42"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="55"/>
+      <c r="I28" s="55"/>
+      <c r="J28" s="55"/>
+      <c r="K28" s="55"/>
+      <c r="L28" s="55"/>
+      <c r="M28" s="55"/>
+      <c r="N28" s="55"/>
+      <c r="O28" s="43"/>
+      <c r="P28" s="55"/>
+      <c r="Q28" s="55"/>
+      <c r="R28" s="55"/>
+      <c r="S28" s="55"/>
+      <c r="T28" s="55"/>
+      <c r="U28" s="55"/>
+      <c r="V28" s="55"/>
+      <c r="W28" s="55"/>
+      <c r="X28" s="55"/>
+      <c r="Y28" s="55"/>
+      <c r="Z28" s="55"/>
+      <c r="AA28" s="55"/>
+      <c r="AB28" s="55"/>
+      <c r="AC28" s="43"/>
+      <c r="AD28" s="43"/>
+      <c r="AE28" s="55"/>
+      <c r="AF28" s="55"/>
+      <c r="AG28" s="55"/>
+      <c r="AH28" s="55"/>
+      <c r="AI28" s="55"/>
+      <c r="AJ28" s="44"/>
+      <c r="AK28" s="42"/>
+      <c r="AL28" s="56"/>
+    </row>
+    <row r="29" s="23" customFormat="1" spans="1:38">
+      <c r="A29" s="60"/>
+      <c r="B29" s="45"/>
+      <c r="C29" s="46"/>
+      <c r="D29" s="41"/>
+      <c r="E29" s="61"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="62"/>
+      <c r="H29" s="52"/>
+      <c r="I29" s="52"/>
+      <c r="J29" s="52"/>
+      <c r="K29" s="52"/>
+      <c r="L29" s="52"/>
+      <c r="M29" s="52"/>
+      <c r="N29" s="52"/>
+      <c r="O29" s="52"/>
+      <c r="P29" s="52"/>
+      <c r="Q29" s="52"/>
+      <c r="R29" s="52"/>
+      <c r="S29" s="43"/>
+      <c r="T29" s="52"/>
+      <c r="U29" s="52"/>
+      <c r="V29" s="63"/>
+      <c r="W29" s="52"/>
+      <c r="X29" s="52"/>
+      <c r="Y29" s="52"/>
+      <c r="Z29" s="52"/>
+      <c r="AA29" s="52"/>
+      <c r="AB29" s="52"/>
+      <c r="AC29" s="64"/>
+      <c r="AD29" s="64"/>
+      <c r="AE29" s="52"/>
+      <c r="AF29" s="52"/>
+      <c r="AG29" s="52"/>
+      <c r="AH29" s="52"/>
+      <c r="AI29" s="62"/>
+      <c r="AJ29" s="53"/>
+      <c r="AK29" s="41"/>
+      <c r="AL29" s="65"/>
+    </row>
+    <row r="30" s="23" customFormat="1" spans="1:38">
+      <c r="A30" s="66" t="s">
         <v>46</v>
       </c>
-      <c r="B30" s="69"/>
-      <c r="C30" s="69"/>
-      <c r="D30" s="69"/>
-      <c r="E30" s="70"/>
-      <c r="F30" s="70"/>
-      <c r="G30" s="70"/>
-      <c r="H30" s="70"/>
-      <c r="I30" s="70"/>
-      <c r="J30" s="70"/>
-      <c r="K30" s="70"/>
-      <c r="L30" s="70"/>
-      <c r="M30" s="70"/>
-      <c r="N30" s="70"/>
-      <c r="O30" s="71"/>
-      <c r="P30" s="70"/>
-      <c r="Q30" s="70"/>
-      <c r="R30" s="70"/>
-      <c r="S30" s="70"/>
-      <c r="T30" s="70"/>
-      <c r="U30" s="70"/>
-      <c r="V30" s="70"/>
-      <c r="W30" s="70"/>
-      <c r="X30" s="70"/>
-      <c r="Y30" s="70"/>
-      <c r="Z30" s="70"/>
-      <c r="AA30" s="70"/>
-      <c r="AB30" s="70"/>
-      <c r="AC30" s="71"/>
-      <c r="AD30" s="71"/>
-      <c r="AE30" s="70"/>
-      <c r="AF30" s="70"/>
-      <c r="AG30" s="70"/>
-      <c r="AH30" s="70"/>
-      <c r="AI30" s="70"/>
-      <c r="AJ30" s="71"/>
-      <c r="AK30" s="69"/>
-      <c r="AL30" s="72"/>
-    </row>
-    <row r="31" s="25" customFormat="1" spans="1:38">
-      <c r="A31" s="73"/>
-      <c r="E31" s="26"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="26"/>
-      <c r="K31" s="26"/>
-      <c r="L31" s="26"/>
-      <c r="M31" s="26"/>
-      <c r="N31" s="26"/>
-      <c r="O31" s="27"/>
-      <c r="P31" s="26"/>
-      <c r="Q31" s="26"/>
-      <c r="R31" s="26"/>
-      <c r="S31" s="26"/>
-      <c r="T31" s="26"/>
-      <c r="U31" s="26"/>
-      <c r="V31" s="26"/>
-      <c r="W31" s="26"/>
-      <c r="X31" s="26"/>
-      <c r="Y31" s="26"/>
-      <c r="Z31" s="26"/>
-      <c r="AA31" s="26"/>
-      <c r="AB31" s="26"/>
-      <c r="AC31" s="27"/>
-      <c r="AD31" s="27"/>
-      <c r="AE31" s="26"/>
-      <c r="AF31" s="26"/>
-      <c r="AG31" s="26"/>
-      <c r="AH31" s="26"/>
-      <c r="AI31" s="26"/>
-      <c r="AJ31" s="27"/>
-      <c r="AL31" s="74"/>
-    </row>
-    <row r="32" s="25" customFormat="1" spans="1:38">
-      <c r="A32" s="73"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
-      <c r="O32" s="27"/>
-      <c r="P32" s="26"/>
-      <c r="Q32" s="26"/>
-      <c r="R32" s="26"/>
-      <c r="S32" s="26"/>
-      <c r="T32" s="26"/>
-      <c r="U32" s="26"/>
-      <c r="V32" s="26"/>
-      <c r="W32" s="26"/>
-      <c r="X32" s="26"/>
-      <c r="Y32" s="26"/>
-      <c r="Z32" s="26"/>
-      <c r="AA32" s="26"/>
-      <c r="AB32" s="26"/>
-      <c r="AC32" s="27"/>
-      <c r="AD32" s="27"/>
-      <c r="AE32" s="26"/>
-      <c r="AF32" s="26"/>
-      <c r="AG32" s="26"/>
-      <c r="AH32" s="26"/>
-      <c r="AI32" s="26"/>
-      <c r="AJ32" s="27"/>
-      <c r="AL32" s="74"/>
-    </row>
-    <row r="33" s="25" customFormat="1" spans="1:38">
-      <c r="A33" s="73"/>
-      <c r="E33" s="26"/>
-      <c r="F33" s="26"/>
-      <c r="G33" s="26"/>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="26"/>
-      <c r="K33" s="26"/>
-      <c r="L33" s="26"/>
-      <c r="M33" s="26"/>
-      <c r="N33" s="26"/>
-      <c r="O33" s="27"/>
-      <c r="P33" s="26"/>
-      <c r="Q33" s="26"/>
-      <c r="R33" s="26"/>
-      <c r="S33" s="26"/>
-      <c r="T33" s="26"/>
-      <c r="U33" s="26"/>
-      <c r="V33" s="26"/>
-      <c r="W33" s="26"/>
-      <c r="X33" s="26"/>
-      <c r="Y33" s="26"/>
-      <c r="Z33" s="26"/>
-      <c r="AA33" s="26"/>
-      <c r="AB33" s="26"/>
-      <c r="AC33" s="27"/>
-      <c r="AD33" s="27"/>
-      <c r="AE33" s="26"/>
-      <c r="AF33" s="26"/>
-      <c r="AG33" s="26"/>
-      <c r="AH33" s="26"/>
-      <c r="AI33" s="26"/>
-      <c r="AJ33" s="27"/>
-      <c r="AL33" s="74"/>
-    </row>
-    <row r="34" s="25" customFormat="1" spans="1:38">
-      <c r="A34" s="73"/>
-      <c r="E34" s="26"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="26"/>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="26"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
-      <c r="N34" s="26"/>
-      <c r="O34" s="27"/>
-      <c r="P34" s="26"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="26"/>
-      <c r="S34" s="26"/>
-      <c r="T34" s="26"/>
-      <c r="U34" s="26"/>
-      <c r="V34" s="26"/>
-      <c r="W34" s="26"/>
-      <c r="X34" s="26"/>
-      <c r="Y34" s="26"/>
-      <c r="Z34" s="26"/>
-      <c r="AA34" s="26"/>
-      <c r="AB34" s="26"/>
-      <c r="AC34" s="27"/>
-      <c r="AD34" s="27"/>
-      <c r="AE34" s="26"/>
-      <c r="AF34" s="26"/>
-      <c r="AG34" s="26"/>
-      <c r="AH34" s="26"/>
-      <c r="AI34" s="26"/>
-      <c r="AJ34" s="27"/>
-      <c r="AL34" s="74"/>
-    </row>
-    <row r="35" s="25" customFormat="1" spans="1:38">
-      <c r="A35" s="75"/>
-      <c r="B35" s="76"/>
-      <c r="C35" s="76"/>
-      <c r="D35" s="76"/>
-      <c r="E35" s="77"/>
-      <c r="F35" s="77"/>
-      <c r="G35" s="77"/>
-      <c r="H35" s="77"/>
-      <c r="I35" s="77"/>
-      <c r="J35" s="77"/>
-      <c r="K35" s="77"/>
-      <c r="L35" s="77"/>
-      <c r="M35" s="77"/>
-      <c r="N35" s="77"/>
-      <c r="O35" s="78"/>
-      <c r="P35" s="77"/>
-      <c r="Q35" s="77"/>
-      <c r="R35" s="77"/>
-      <c r="S35" s="77"/>
-      <c r="T35" s="77"/>
-      <c r="U35" s="77"/>
-      <c r="V35" s="77"/>
-      <c r="W35" s="77"/>
-      <c r="X35" s="77"/>
-      <c r="Y35" s="77"/>
-      <c r="Z35" s="77"/>
-      <c r="AA35" s="77"/>
-      <c r="AB35" s="77"/>
-      <c r="AC35" s="78"/>
-      <c r="AD35" s="78"/>
-      <c r="AE35" s="77"/>
-      <c r="AF35" s="77"/>
-      <c r="AG35" s="77"/>
-      <c r="AH35" s="77"/>
-      <c r="AI35" s="77"/>
-      <c r="AJ35" s="78"/>
-      <c r="AK35" s="76"/>
-      <c r="AL35" s="79"/>
-    </row>
-    <row r="36" s="25" customFormat="1" spans="1:38">
-      <c r="A36" s="68" t="s">
+      <c r="B30" s="67"/>
+      <c r="C30" s="67"/>
+      <c r="D30" s="67"/>
+      <c r="E30" s="68"/>
+      <c r="F30" s="68"/>
+      <c r="G30" s="68"/>
+      <c r="H30" s="68"/>
+      <c r="I30" s="68"/>
+      <c r="J30" s="68"/>
+      <c r="K30" s="68"/>
+      <c r="L30" s="68"/>
+      <c r="M30" s="68"/>
+      <c r="N30" s="68"/>
+      <c r="O30" s="69"/>
+      <c r="P30" s="68"/>
+      <c r="Q30" s="68"/>
+      <c r="R30" s="68"/>
+      <c r="S30" s="68"/>
+      <c r="T30" s="68"/>
+      <c r="U30" s="68"/>
+      <c r="V30" s="68"/>
+      <c r="W30" s="68"/>
+      <c r="X30" s="68"/>
+      <c r="Y30" s="68"/>
+      <c r="Z30" s="68"/>
+      <c r="AA30" s="68"/>
+      <c r="AB30" s="68"/>
+      <c r="AC30" s="69"/>
+      <c r="AD30" s="69"/>
+      <c r="AE30" s="68"/>
+      <c r="AF30" s="68"/>
+      <c r="AG30" s="68"/>
+      <c r="AH30" s="68"/>
+      <c r="AI30" s="68"/>
+      <c r="AJ30" s="69"/>
+      <c r="AK30" s="67"/>
+      <c r="AL30" s="70"/>
+    </row>
+    <row r="31" s="23" customFormat="1" spans="1:38">
+      <c r="A31" s="71"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="24"/>
+      <c r="I31" s="24"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="24"/>
+      <c r="L31" s="24"/>
+      <c r="M31" s="24"/>
+      <c r="N31" s="24"/>
+      <c r="O31" s="25"/>
+      <c r="P31" s="24"/>
+      <c r="Q31" s="24"/>
+      <c r="R31" s="24"/>
+      <c r="S31" s="24"/>
+      <c r="T31" s="24"/>
+      <c r="U31" s="24"/>
+      <c r="V31" s="24"/>
+      <c r="W31" s="24"/>
+      <c r="X31" s="24"/>
+      <c r="Y31" s="24"/>
+      <c r="Z31" s="24"/>
+      <c r="AA31" s="24"/>
+      <c r="AB31" s="24"/>
+      <c r="AC31" s="25"/>
+      <c r="AD31" s="25"/>
+      <c r="AE31" s="24"/>
+      <c r="AF31" s="24"/>
+      <c r="AG31" s="24"/>
+      <c r="AH31" s="24"/>
+      <c r="AI31" s="24"/>
+      <c r="AJ31" s="25"/>
+      <c r="AL31" s="72"/>
+    </row>
+    <row r="32" s="23" customFormat="1" spans="1:38">
+      <c r="A32" s="71"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="24"/>
+      <c r="L32" s="24"/>
+      <c r="M32" s="24"/>
+      <c r="N32" s="24"/>
+      <c r="O32" s="25"/>
+      <c r="P32" s="24"/>
+      <c r="Q32" s="24"/>
+      <c r="R32" s="24"/>
+      <c r="S32" s="24"/>
+      <c r="T32" s="24"/>
+      <c r="U32" s="24"/>
+      <c r="V32" s="24"/>
+      <c r="W32" s="24"/>
+      <c r="X32" s="24"/>
+      <c r="Y32" s="24"/>
+      <c r="Z32" s="24"/>
+      <c r="AA32" s="24"/>
+      <c r="AB32" s="24"/>
+      <c r="AC32" s="25"/>
+      <c r="AD32" s="25"/>
+      <c r="AE32" s="24"/>
+      <c r="AF32" s="24"/>
+      <c r="AG32" s="24"/>
+      <c r="AH32" s="24"/>
+      <c r="AI32" s="24"/>
+      <c r="AJ32" s="25"/>
+      <c r="AL32" s="72"/>
+    </row>
+    <row r="33" s="23" customFormat="1" spans="1:38">
+      <c r="A33" s="71"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="24"/>
+      <c r="I33" s="24"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="24"/>
+      <c r="L33" s="24"/>
+      <c r="M33" s="24"/>
+      <c r="N33" s="24"/>
+      <c r="O33" s="25"/>
+      <c r="P33" s="24"/>
+      <c r="Q33" s="24"/>
+      <c r="R33" s="24"/>
+      <c r="S33" s="24"/>
+      <c r="T33" s="24"/>
+      <c r="U33" s="24"/>
+      <c r="V33" s="24"/>
+      <c r="W33" s="24"/>
+      <c r="X33" s="24"/>
+      <c r="Y33" s="24"/>
+      <c r="Z33" s="24"/>
+      <c r="AA33" s="24"/>
+      <c r="AB33" s="24"/>
+      <c r="AC33" s="25"/>
+      <c r="AD33" s="25"/>
+      <c r="AE33" s="24"/>
+      <c r="AF33" s="24"/>
+      <c r="AG33" s="24"/>
+      <c r="AH33" s="24"/>
+      <c r="AI33" s="24"/>
+      <c r="AJ33" s="25"/>
+      <c r="AL33" s="72"/>
+    </row>
+    <row r="34" s="23" customFormat="1" spans="1:38">
+      <c r="A34" s="71"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="24"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="24"/>
+      <c r="N34" s="24"/>
+      <c r="O34" s="25"/>
+      <c r="P34" s="24"/>
+      <c r="Q34" s="24"/>
+      <c r="R34" s="24"/>
+      <c r="S34" s="24"/>
+      <c r="T34" s="24"/>
+      <c r="U34" s="24"/>
+      <c r="V34" s="24"/>
+      <c r="W34" s="24"/>
+      <c r="X34" s="24"/>
+      <c r="Y34" s="24"/>
+      <c r="Z34" s="24"/>
+      <c r="AA34" s="24"/>
+      <c r="AB34" s="24"/>
+      <c r="AC34" s="25"/>
+      <c r="AD34" s="25"/>
+      <c r="AE34" s="24"/>
+      <c r="AF34" s="24"/>
+      <c r="AG34" s="24"/>
+      <c r="AH34" s="24"/>
+      <c r="AI34" s="24"/>
+      <c r="AJ34" s="25"/>
+      <c r="AL34" s="72"/>
+    </row>
+    <row r="35" s="23" customFormat="1" spans="1:38">
+      <c r="A35" s="73"/>
+      <c r="B35" s="74"/>
+      <c r="C35" s="74"/>
+      <c r="D35" s="74"/>
+      <c r="E35" s="75"/>
+      <c r="F35" s="75"/>
+      <c r="G35" s="75"/>
+      <c r="H35" s="75"/>
+      <c r="I35" s="75"/>
+      <c r="J35" s="75"/>
+      <c r="K35" s="75"/>
+      <c r="L35" s="75"/>
+      <c r="M35" s="75"/>
+      <c r="N35" s="75"/>
+      <c r="O35" s="76"/>
+      <c r="P35" s="75"/>
+      <c r="Q35" s="75"/>
+      <c r="R35" s="75"/>
+      <c r="S35" s="75"/>
+      <c r="T35" s="75"/>
+      <c r="U35" s="75"/>
+      <c r="V35" s="75"/>
+      <c r="W35" s="75"/>
+      <c r="X35" s="75"/>
+      <c r="Y35" s="75"/>
+      <c r="Z35" s="75"/>
+      <c r="AA35" s="75"/>
+      <c r="AB35" s="75"/>
+      <c r="AC35" s="76"/>
+      <c r="AD35" s="76"/>
+      <c r="AE35" s="75"/>
+      <c r="AF35" s="75"/>
+      <c r="AG35" s="75"/>
+      <c r="AH35" s="75"/>
+      <c r="AI35" s="75"/>
+      <c r="AJ35" s="76"/>
+      <c r="AK35" s="74"/>
+      <c r="AL35" s="77"/>
+    </row>
+    <row r="36" s="23" customFormat="1" spans="1:38">
+      <c r="A36" s="66" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="69"/>
-      <c r="C36" s="69"/>
-      <c r="D36" s="69"/>
-      <c r="E36" s="70"/>
-      <c r="F36" s="70"/>
-      <c r="G36" s="70"/>
-      <c r="H36" s="70"/>
-      <c r="I36" s="70"/>
-      <c r="J36" s="70"/>
-      <c r="K36" s="70"/>
-      <c r="L36" s="70"/>
-      <c r="M36" s="70"/>
-      <c r="N36" s="70"/>
-      <c r="O36" s="71"/>
-      <c r="P36" s="70"/>
-      <c r="Q36" s="70"/>
-      <c r="R36" s="70"/>
-      <c r="S36" s="70"/>
-      <c r="T36" s="70"/>
-      <c r="U36" s="70"/>
-      <c r="V36" s="70"/>
-      <c r="W36" s="70"/>
-      <c r="X36" s="70"/>
-      <c r="Y36" s="70"/>
-      <c r="Z36" s="70"/>
-      <c r="AA36" s="70"/>
-      <c r="AB36" s="70"/>
-      <c r="AC36" s="71"/>
-      <c r="AD36" s="71"/>
-      <c r="AE36" s="70"/>
-      <c r="AF36" s="70"/>
-      <c r="AG36" s="70"/>
-      <c r="AH36" s="70"/>
-      <c r="AI36" s="70"/>
-      <c r="AJ36" s="71"/>
-      <c r="AK36" s="69"/>
-      <c r="AL36" s="72"/>
-    </row>
-    <row r="37" s="25" customFormat="1" spans="1:38">
-      <c r="A37" s="73"/>
-      <c r="E37" s="26"/>
-      <c r="F37" s="26"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
-      <c r="K37" s="26"/>
-      <c r="L37" s="26"/>
-      <c r="M37" s="26"/>
-      <c r="N37" s="26"/>
-      <c r="O37" s="27"/>
-      <c r="P37" s="26"/>
-      <c r="Q37" s="26"/>
-      <c r="R37" s="26"/>
-      <c r="S37" s="26"/>
-      <c r="T37" s="26"/>
-      <c r="U37" s="26"/>
-      <c r="V37" s="26"/>
-      <c r="W37" s="26"/>
-      <c r="X37" s="26"/>
-      <c r="Y37" s="26"/>
-      <c r="Z37" s="26"/>
-      <c r="AA37" s="26"/>
-      <c r="AB37" s="26"/>
-      <c r="AC37" s="27"/>
-      <c r="AD37" s="27"/>
-      <c r="AE37" s="26"/>
-      <c r="AF37" s="26"/>
-      <c r="AG37" s="26"/>
-      <c r="AH37" s="26"/>
-      <c r="AI37" s="26"/>
-      <c r="AJ37" s="27"/>
-      <c r="AL37" s="74"/>
-    </row>
-    <row r="38" s="25" customFormat="1" spans="1:38">
-      <c r="A38" s="75"/>
-      <c r="B38" s="76"/>
-      <c r="C38" s="76"/>
-      <c r="D38" s="76"/>
-      <c r="E38" s="77"/>
-      <c r="F38" s="77"/>
-      <c r="G38" s="77"/>
-      <c r="H38" s="77"/>
-      <c r="I38" s="77"/>
-      <c r="J38" s="77"/>
-      <c r="K38" s="77"/>
-      <c r="L38" s="77"/>
-      <c r="M38" s="77"/>
-      <c r="N38" s="77"/>
-      <c r="O38" s="78"/>
-      <c r="P38" s="77"/>
-      <c r="Q38" s="77"/>
-      <c r="R38" s="77"/>
-      <c r="S38" s="77"/>
-      <c r="T38" s="77"/>
-      <c r="U38" s="77"/>
-      <c r="V38" s="77"/>
-      <c r="W38" s="77"/>
-      <c r="X38" s="77"/>
-      <c r="Y38" s="77"/>
-      <c r="Z38" s="77"/>
-      <c r="AA38" s="77"/>
-      <c r="AB38" s="77"/>
-      <c r="AC38" s="78"/>
-      <c r="AD38" s="78"/>
-      <c r="AE38" s="77"/>
-      <c r="AF38" s="77"/>
-      <c r="AG38" s="77"/>
-      <c r="AH38" s="77"/>
-      <c r="AI38" s="77"/>
-      <c r="AJ38" s="78"/>
-      <c r="AK38" s="76"/>
-      <c r="AL38" s="79"/>
+      <c r="B36" s="67"/>
+      <c r="C36" s="67"/>
+      <c r="D36" s="67"/>
+      <c r="E36" s="68"/>
+      <c r="F36" s="68"/>
+      <c r="G36" s="68"/>
+      <c r="H36" s="68"/>
+      <c r="I36" s="68"/>
+      <c r="J36" s="68"/>
+      <c r="K36" s="68"/>
+      <c r="L36" s="68"/>
+      <c r="M36" s="68"/>
+      <c r="N36" s="68"/>
+      <c r="O36" s="69"/>
+      <c r="P36" s="68"/>
+      <c r="Q36" s="68"/>
+      <c r="R36" s="68"/>
+      <c r="S36" s="68"/>
+      <c r="T36" s="68"/>
+      <c r="U36" s="68"/>
+      <c r="V36" s="68"/>
+      <c r="W36" s="68"/>
+      <c r="X36" s="68"/>
+      <c r="Y36" s="68"/>
+      <c r="Z36" s="68"/>
+      <c r="AA36" s="68"/>
+      <c r="AB36" s="68"/>
+      <c r="AC36" s="69"/>
+      <c r="AD36" s="69"/>
+      <c r="AE36" s="68"/>
+      <c r="AF36" s="68"/>
+      <c r="AG36" s="68"/>
+      <c r="AH36" s="68"/>
+      <c r="AI36" s="68"/>
+      <c r="AJ36" s="69"/>
+      <c r="AK36" s="67"/>
+      <c r="AL36" s="70"/>
+    </row>
+    <row r="37" s="23" customFormat="1" spans="1:38">
+      <c r="A37" s="71"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="24"/>
+      <c r="I37" s="24"/>
+      <c r="J37" s="24"/>
+      <c r="K37" s="24"/>
+      <c r="L37" s="24"/>
+      <c r="M37" s="24"/>
+      <c r="N37" s="24"/>
+      <c r="O37" s="25"/>
+      <c r="P37" s="24"/>
+      <c r="Q37" s="24"/>
+      <c r="R37" s="24"/>
+      <c r="S37" s="24"/>
+      <c r="T37" s="24"/>
+      <c r="U37" s="24"/>
+      <c r="V37" s="24"/>
+      <c r="W37" s="24"/>
+      <c r="X37" s="24"/>
+      <c r="Y37" s="24"/>
+      <c r="Z37" s="24"/>
+      <c r="AA37" s="24"/>
+      <c r="AB37" s="24"/>
+      <c r="AC37" s="25"/>
+      <c r="AD37" s="25"/>
+      <c r="AE37" s="24"/>
+      <c r="AF37" s="24"/>
+      <c r="AG37" s="24"/>
+      <c r="AH37" s="24"/>
+      <c r="AI37" s="24"/>
+      <c r="AJ37" s="25"/>
+      <c r="AL37" s="72"/>
+    </row>
+    <row r="38" s="23" customFormat="1" spans="1:38">
+      <c r="A38" s="73"/>
+      <c r="B38" s="74"/>
+      <c r="C38" s="74"/>
+      <c r="D38" s="74"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="75"/>
+      <c r="G38" s="75"/>
+      <c r="H38" s="75"/>
+      <c r="I38" s="75"/>
+      <c r="J38" s="75"/>
+      <c r="K38" s="75"/>
+      <c r="L38" s="75"/>
+      <c r="M38" s="75"/>
+      <c r="N38" s="75"/>
+      <c r="O38" s="76"/>
+      <c r="P38" s="75"/>
+      <c r="Q38" s="75"/>
+      <c r="R38" s="75"/>
+      <c r="S38" s="75"/>
+      <c r="T38" s="75"/>
+      <c r="U38" s="75"/>
+      <c r="V38" s="75"/>
+      <c r="W38" s="75"/>
+      <c r="X38" s="75"/>
+      <c r="Y38" s="75"/>
+      <c r="Z38" s="75"/>
+      <c r="AA38" s="75"/>
+      <c r="AB38" s="75"/>
+      <c r="AC38" s="76"/>
+      <c r="AD38" s="76"/>
+      <c r="AE38" s="75"/>
+      <c r="AF38" s="75"/>
+      <c r="AG38" s="75"/>
+      <c r="AH38" s="75"/>
+      <c r="AI38" s="75"/>
+      <c r="AJ38" s="76"/>
+      <c r="AK38" s="74"/>
+      <c r="AL38" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="63">
@@ -3620,7 +3608,7 @@
   <pageMargins left="0.357638888888889" right="0.357638888888889" top="0.802777777777778" bottom="0.2125" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="90" orientation="landscape" blackAndWhite="1" horizontalDpi="600"/>
   <headerFooter/>
-  <rowBreaks count="9" manualBreakCount="9">
+  <rowBreaks count="1" manualBreakCount="1">
     <brk id="38" max="255" man="1"/>
   </rowBreaks>
 </worksheet>
@@ -3632,7 +3620,7 @@
     <tabColor rgb="FFFFC000"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB27"/>
+  <dimension ref="A1:AB25"/>
   <sheetFormatPr defaultColWidth="8.19166666666667" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="4.06666666666667" style="1" customWidth="1"/>
@@ -3740,19 +3728,19 @@
       <c r="C4" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="81" t="s">
+      <c r="D4" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="81" t="s">
+      <c r="E4" s="79" t="s">
         <v>62</v>
       </c>
       <c r="F4" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="G4" s="82" t="s">
+      <c r="G4" s="80" t="s">
         <v>64</v>
       </c>
-      <c r="H4" s="82" t="s">
+      <c r="H4" s="80" t="s">
         <v>65</v>
       </c>
       <c r="I4" s="16">
@@ -4088,94 +4076,48 @@
       <c r="L23" s="16"/>
       <c r="M23" s="17"/>
     </row>
-    <row r="24" ht="21" customHeight="1" spans="1:28">
-      <c r="A24" s="15" t="s">
+    <row r="24" s="2" customFormat="1" ht="30" customHeight="1" spans="1:28">
+      <c r="A24" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
-      <c r="I24" s="16">
-        <f>SUM(I4:I23)</f>
-        <v>38</v>
-      </c>
-      <c r="J24" s="15"/>
-      <c r="K24" s="18">
-        <f>SUM(K4:K23)</f>
-        <v>22800</v>
-      </c>
-      <c r="L24" s="16"/>
-      <c r="M24" s="17"/>
-    </row>
-    <row r="25" ht="19.05" customHeight="1" spans="1:28">
-      <c r="A25" s="12" t="s">
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="16">
-        <f>I24</f>
-        <v>38</v>
-      </c>
-      <c r="J25" s="15"/>
-      <c r="K25" s="18">
-        <f>K24</f>
-        <v>22800</v>
-      </c>
-      <c r="L25" s="19"/>
-      <c r="M25" s="19"/>
-    </row>
-    <row r="26" s="2" customFormat="1" ht="30" customHeight="1" spans="1:28">
-      <c r="A26" s="20" t="s">
+      <c r="F24" s="18"/>
+      <c r="G24" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20" t="s">
+      <c r="I24" s="20"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="F26" s="20"/>
-      <c r="G26" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="I26" s="22"/>
-      <c r="J26" s="20"/>
-      <c r="K26" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="L26" s="20"/>
-      <c r="M26" s="23"/>
-      <c r="N26" s="24"/>
-      <c r="O26" s="24"/>
-      <c r="P26" s="24"/>
-      <c r="Q26" s="24"/>
-      <c r="R26" s="24"/>
-      <c r="S26" s="24"/>
-      <c r="T26" s="24"/>
-      <c r="U26" s="24"/>
-      <c r="V26" s="24"/>
-      <c r="W26" s="24"/>
-      <c r="X26" s="24"/>
-      <c r="Y26" s="24"/>
-      <c r="Z26" s="24"/>
-      <c r="AA26" s="24"/>
-      <c r="AB26" s="24"/>
-    </row>
-    <row r="27" s="1" customFormat="1" spans="1:28">
-      <c r="I27" s="3"/>
+      <c r="L24" s="18"/>
+      <c r="M24" s="21"/>
+      <c r="N24" s="22"/>
+      <c r="O24" s="22"/>
+      <c r="P24" s="22"/>
+      <c r="Q24" s="22"/>
+      <c r="R24" s="22"/>
+      <c r="S24" s="22"/>
+      <c r="T24" s="22"/>
+      <c r="U24" s="22"/>
+      <c r="V24" s="22"/>
+      <c r="W24" s="22"/>
+      <c r="X24" s="22"/>
+      <c r="Y24" s="22"/>
+      <c r="Z24" s="22"/>
+      <c r="AA24" s="22"/>
+      <c r="AB24" s="22"/>
+    </row>
+    <row r="25" s="1" customFormat="1" spans="1:28">
+      <c r="I25" s="3"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:Z26" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A3:Z24" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <mergeCells count="3">
@@ -4187,9 +4129,8 @@
   <pageMargins left="0.357638888888889" right="0.357638888888889" top="0.802777777777778" bottom="0.60625" header="0.511805555555556" footer="0.511805555555556"/>
   <pageSetup paperSize="9" scale="95" fitToHeight="0" orientation="landscape" blackAndWhite="1" horizontalDpi="600"/>
   <headerFooter alignWithMargins="0" scaleWithDoc="0"/>
-  <rowBreaks count="5" manualBreakCount="5">
+  <rowBreaks count="2" manualBreakCount="2">
     <brk id="24" max="255" man="1"/>
-    <brk id="26" max="255" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>